<commit_message>
some fixes in parameter files
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\modelX\data\prod_parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\data\prod_parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="13" r:id="rId1"/>
@@ -56,13 +56,13 @@
   </definedNames>
   <calcPr calcId="162913" iterate="1"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId12"/>
+    <pivotCache cacheId="1" r:id="rId12"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2435" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="435">
   <si>
     <t>value</t>
   </si>
@@ -1371,6 +1371,15 @@
   <si>
     <t>breeding bulls</t>
   </si>
+  <si>
+    <t>Maximum share of grazing in semi-natural grasslands</t>
+  </si>
+  <si>
+    <t>max_sng_grazing</t>
+  </si>
+  <si>
+    <t>This parameter specifies the maximum share of grazing demand that can be met from grazing in semi-natural grasslands</t>
+  </si>
 </sst>
 </file>
 
@@ -1383,7 +1392,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1628,6 +1637,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="40">
@@ -2220,7 +2236,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2333,7 +2349,6 @@
     <xf numFmtId="2" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -2473,6 +2488,8 @@
     <xf numFmtId="167" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -13985,7 +14002,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L3:O43" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField axis="axisRow" showAll="0">
@@ -14477,7 +14494,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="109" t="s">
         <v>331</v>
       </c>
     </row>
@@ -14498,48 +14515,48 @@
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="140" t="s">
+      <c r="A3" s="139" t="s">
         <v>359</v>
       </c>
-      <c r="B3" s="140"/>
+      <c r="B3" s="139"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="137" t="s">
+      <c r="A4" s="136" t="s">
         <v>360</v>
       </c>
-      <c r="B4" s="137">
+      <c r="B4" s="136">
         <v>0.99434308508956182</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="136" t="s">
         <v>361</v>
       </c>
-      <c r="B5" s="137">
+      <c r="B5" s="136">
         <v>0.98871817086542757</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="137" t="s">
+      <c r="A6" s="136" t="s">
         <v>362</v>
       </c>
-      <c r="B6" s="142">
+      <c r="B6" s="141">
         <v>0.9876437109478492</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="137" t="s">
+      <c r="A7" s="136" t="s">
         <v>363</v>
       </c>
-      <c r="B7" s="137">
+      <c r="B7" s="136">
         <v>0.64295634155271764</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="138" t="s">
+      <c r="A8" s="137" t="s">
         <v>364</v>
       </c>
-      <c r="B8" s="138">
+      <c r="B8" s="137">
         <v>24</v>
       </c>
     </row>
@@ -14549,185 +14566,185 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="139"/>
-      <c r="B11" s="139" t="s">
+      <c r="A11" s="138"/>
+      <c r="B11" s="138" t="s">
         <v>369</v>
       </c>
-      <c r="C11" s="139" t="s">
+      <c r="C11" s="138" t="s">
         <v>370</v>
       </c>
-      <c r="D11" s="139" t="s">
+      <c r="D11" s="138" t="s">
         <v>371</v>
       </c>
-      <c r="E11" s="139" t="s">
+      <c r="E11" s="138" t="s">
         <v>372</v>
       </c>
-      <c r="F11" s="139" t="s">
+      <c r="F11" s="138" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="137" t="s">
+      <c r="A12" s="136" t="s">
         <v>366</v>
       </c>
-      <c r="B12" s="137">
+      <c r="B12" s="136">
         <v>2</v>
       </c>
-      <c r="C12" s="137">
+      <c r="C12" s="136">
         <v>760.80833333333317</v>
       </c>
-      <c r="D12" s="137">
+      <c r="D12" s="136">
         <v>380.40416666666658</v>
       </c>
-      <c r="E12" s="137">
+      <c r="E12" s="136">
         <v>920.20014398848559</v>
       </c>
-      <c r="F12" s="137">
+      <c r="F12" s="136">
         <v>3.5480108451103033E-21</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="137" t="s">
+      <c r="A13" s="136" t="s">
         <v>367</v>
       </c>
-      <c r="B13" s="137">
+      <c r="B13" s="136">
         <v>21</v>
       </c>
-      <c r="C13" s="137">
+      <c r="C13" s="136">
         <v>8.6812499999999542</v>
       </c>
-      <c r="D13" s="137">
+      <c r="D13" s="136">
         <v>0.41339285714285495</v>
       </c>
-      <c r="E13" s="137"/>
-      <c r="F13" s="137"/>
+      <c r="E13" s="136"/>
+      <c r="F13" s="136"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="138" t="s">
+      <c r="A14" s="137" t="s">
         <v>317</v>
       </c>
-      <c r="B14" s="138">
+      <c r="B14" s="137">
         <v>23</v>
       </c>
-      <c r="C14" s="138">
+      <c r="C14" s="137">
         <v>769.48958333333314</v>
       </c>
-      <c r="D14" s="138"/>
-      <c r="E14" s="138"/>
-      <c r="F14" s="138"/>
+      <c r="D14" s="137"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="137"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="139"/>
-      <c r="B16" s="139" t="s">
+      <c r="A16" s="138"/>
+      <c r="B16" s="138" t="s">
         <v>374</v>
       </c>
-      <c r="C16" s="139" t="s">
+      <c r="C16" s="138" t="s">
         <v>363</v>
       </c>
-      <c r="D16" s="139" t="s">
+      <c r="D16" s="138" t="s">
         <v>375</v>
       </c>
-      <c r="E16" s="139" t="s">
+      <c r="E16" s="138" t="s">
         <v>376</v>
       </c>
-      <c r="F16" s="139" t="s">
+      <c r="F16" s="138" t="s">
         <v>377</v>
       </c>
-      <c r="G16" s="139" t="s">
+      <c r="G16" s="138" t="s">
         <v>378</v>
       </c>
-      <c r="H16" s="139" t="s">
+      <c r="H16" s="138" t="s">
         <v>379</v>
       </c>
-      <c r="I16" s="139" t="s">
+      <c r="I16" s="138" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="137" t="s">
+      <c r="A17" s="136" t="s">
         <v>368</v>
       </c>
-      <c r="B17" s="137">
+      <c r="B17" s="136">
         <v>-0.40773809523810023</v>
       </c>
-      <c r="C17" s="137">
+      <c r="C17" s="136">
         <v>0.46902457944381531</v>
       </c>
-      <c r="D17" s="137">
+      <c r="D17" s="136">
         <v>-0.86933204166316702</v>
       </c>
-      <c r="E17" s="137">
+      <c r="E17" s="136">
         <v>0.3944933503705087</v>
       </c>
-      <c r="F17" s="137">
+      <c r="F17" s="136">
         <v>-1.383128104167036</v>
       </c>
-      <c r="G17" s="137">
+      <c r="G17" s="136">
         <v>0.56765191369083567</v>
       </c>
-      <c r="H17" s="137">
+      <c r="H17" s="136">
         <v>-1.383128104167036</v>
       </c>
-      <c r="I17" s="137">
+      <c r="I17" s="136">
         <v>0.56765191369083567</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="137" t="s">
+      <c r="A18" s="136" t="s">
         <v>349</v>
       </c>
-      <c r="B18" s="137">
+      <c r="B18" s="136">
         <v>0.16892857142857148</v>
       </c>
-      <c r="C18" s="137">
+      <c r="C18" s="136">
         <v>7.6847981397678419E-3</v>
       </c>
-      <c r="D18" s="137">
+      <c r="D18" s="136">
         <v>21.982174203690253</v>
       </c>
-      <c r="E18" s="137">
+      <c r="E18" s="136">
         <v>5.622260089430527E-16</v>
       </c>
-      <c r="F18" s="137">
+      <c r="F18" s="136">
         <v>0.15294715882317275</v>
       </c>
-      <c r="G18" s="137">
+      <c r="G18" s="136">
         <v>0.18490998403397021</v>
       </c>
-      <c r="H18" s="137">
+      <c r="H18" s="136">
         <v>0.15294715882317275</v>
       </c>
-      <c r="I18" s="137">
+      <c r="I18" s="136">
         <v>0.18490998403397021</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="138" t="s">
+      <c r="A19" s="137" t="s">
         <v>356</v>
       </c>
-      <c r="B19" s="138">
+      <c r="B19" s="137">
         <v>1.3076190476190479E-2</v>
       </c>
-      <c r="C19" s="138">
+      <c r="C19" s="137">
         <v>3.549456219730319E-4</v>
       </c>
-      <c r="D19" s="138">
+      <c r="D19" s="137">
         <v>36.839982427460349</v>
       </c>
-      <c r="E19" s="138">
+      <c r="E19" s="137">
         <v>1.4430475578158989E-20</v>
       </c>
-      <c r="F19" s="138">
+      <c r="F19" s="137">
         <v>1.2338040646609885E-2</v>
       </c>
-      <c r="G19" s="138">
+      <c r="G19" s="137">
         <v>1.3814340305771073E-2</v>
       </c>
-      <c r="H19" s="138">
+      <c r="H19" s="137">
         <v>1.2338040646609885E-2</v>
       </c>
-      <c r="I19" s="138">
+      <c r="I19" s="137">
         <v>1.3814340305771073E-2</v>
       </c>
     </row>
@@ -14738,352 +14755,352 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="139" t="s">
+      <c r="A25" s="138" t="s">
         <v>382</v>
       </c>
-      <c r="B25" s="139" t="s">
+      <c r="B25" s="138" t="s">
         <v>383</v>
       </c>
-      <c r="C25" s="139" t="s">
+      <c r="C25" s="138" t="s">
         <v>384</v>
       </c>
-      <c r="D25" s="139" t="s">
+      <c r="D25" s="138" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="137">
+      <c r="A26" s="136">
         <v>1</v>
       </c>
-      <c r="B26" s="137">
+      <c r="B26" s="136">
         <v>4.6601190476190446</v>
       </c>
-      <c r="C26" s="137">
+      <c r="C26" s="136">
         <v>1.3398809523809554</v>
       </c>
-      <c r="D26" s="137">
+      <c r="D26" s="136">
         <v>2.1809163068088218</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="137">
+      <c r="A27" s="136">
         <v>2</v>
       </c>
-      <c r="B27" s="137">
+      <c r="B27" s="136">
         <v>6.3494047619047596</v>
       </c>
-      <c r="C27" s="137">
+      <c r="C27" s="136">
         <v>0.65059523809524045</v>
       </c>
-      <c r="D27" s="137">
+      <c r="D27" s="136">
         <v>1.0589700236970436</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="137">
+      <c r="A28" s="136">
         <v>3</v>
       </c>
-      <c r="B28" s="137">
+      <c r="B28" s="136">
         <v>8.0386904761904745</v>
       </c>
-      <c r="C28" s="137">
+      <c r="C28" s="136">
         <v>0.4613095238095255</v>
       </c>
-      <c r="D28" s="137">
+      <c r="D28" s="136">
         <v>0.75087078532955975</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="137">
+      <c r="A29" s="136">
         <v>4</v>
       </c>
-      <c r="B29" s="137">
+      <c r="B29" s="136">
         <v>9.7279761904761894</v>
       </c>
-      <c r="C29" s="137">
+      <c r="C29" s="136">
         <v>0.27202380952381056</v>
       </c>
-      <c r="D29" s="137">
+      <c r="D29" s="136">
         <v>0.44277154696207599</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="137">
+      <c r="A30" s="136">
         <v>5</v>
       </c>
-      <c r="B30" s="137">
+      <c r="B30" s="136">
         <v>11.417261904761904</v>
       </c>
-      <c r="C30" s="137">
+      <c r="C30" s="136">
         <v>8.273809523809561E-2</v>
       </c>
-      <c r="D30" s="137">
+      <c r="D30" s="136">
         <v>0.13467230859459212</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="137">
+      <c r="A31" s="136">
         <v>6</v>
       </c>
-      <c r="B31" s="137">
+      <c r="B31" s="136">
         <v>13.106547619047619</v>
       </c>
-      <c r="C31" s="137">
+      <c r="C31" s="136">
         <v>-0.10654761904761934</v>
       </c>
-      <c r="D31" s="137">
+      <c r="D31" s="136">
         <v>-0.1734269297728917</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="137">
+      <c r="A32" s="136">
         <v>7</v>
       </c>
-      <c r="B32" s="137">
+      <c r="B32" s="136">
         <v>7.9291666666666645</v>
       </c>
-      <c r="C32" s="137">
+      <c r="C32" s="136">
         <v>7.0833333333335524E-2</v>
       </c>
-      <c r="D32" s="137">
+      <c r="D32" s="136">
         <v>0.11529499800544522</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="137">
+      <c r="A33" s="136">
         <v>8</v>
       </c>
-      <c r="B33" s="137">
+      <c r="B33" s="136">
         <v>9.6184523809523803</v>
       </c>
-      <c r="C33" s="137">
+      <c r="C33" s="136">
         <v>-0.11845238095238031</v>
       </c>
-      <c r="D33" s="137">
+      <c r="D33" s="136">
         <v>-0.19280424036204005</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="137">
+      <c r="A34" s="136">
         <v>9</v>
       </c>
-      <c r="B34" s="137">
+      <c r="B34" s="136">
         <v>11.307738095238093</v>
       </c>
-      <c r="C34" s="137">
+      <c r="C34" s="136">
         <v>-0.30773809523809348</v>
       </c>
-      <c r="D34" s="137">
+      <c r="D34" s="136">
         <v>-0.50090347872952101</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="137">
+      <c r="A35" s="136">
         <v>10</v>
       </c>
-      <c r="B35" s="137">
+      <c r="B35" s="136">
         <v>12.99702380952381</v>
       </c>
-      <c r="C35" s="137">
+      <c r="C35" s="136">
         <v>-0.4970238095238102</v>
       </c>
-      <c r="D35" s="137">
+      <c r="D35" s="136">
         <v>-0.80900271709700777</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="137">
+      <c r="A36" s="136">
         <v>11</v>
       </c>
-      <c r="B36" s="137">
+      <c r="B36" s="136">
         <v>14.686309523809523</v>
       </c>
-      <c r="C36" s="137">
+      <c r="C36" s="136">
         <v>-0.68630952380952337</v>
       </c>
-      <c r="D36" s="137">
+      <c r="D36" s="136">
         <v>-1.1171019554644888</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="137">
+      <c r="A37" s="136">
         <v>12</v>
       </c>
-      <c r="B37" s="137">
+      <c r="B37" s="136">
         <v>16.37559523809524</v>
       </c>
-      <c r="C37" s="137">
+      <c r="C37" s="136">
         <v>-0.37559523809524009</v>
       </c>
-      <c r="D37" s="137">
+      <c r="D37" s="136">
         <v>-0.61135414908768126</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="137">
+      <c r="A38" s="136">
         <v>13</v>
       </c>
-      <c r="B38" s="137">
+      <c r="B38" s="136">
         <v>11.198214285714284</v>
       </c>
-      <c r="C38" s="137">
+      <c r="C38" s="136">
         <v>-0.19821428571428434</v>
       </c>
-      <c r="D38" s="137">
+      <c r="D38" s="136">
         <v>-0.32263222130934294</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="137">
+      <c r="A39" s="136">
         <v>14</v>
       </c>
-      <c r="B39" s="137">
+      <c r="B39" s="136">
         <v>12.887499999999999</v>
       </c>
-      <c r="C39" s="137">
+      <c r="C39" s="136">
         <v>-0.38749999999999929</v>
       </c>
-      <c r="D39" s="137">
+      <c r="D39" s="136">
         <v>-0.63073145967682676</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="137">
+      <c r="A40" s="136">
         <v>15</v>
       </c>
-      <c r="B40" s="137">
+      <c r="B40" s="136">
         <v>14.576785714285714</v>
       </c>
-      <c r="C40" s="137">
+      <c r="C40" s="136">
         <v>-0.57678571428571423</v>
       </c>
-      <c r="D40" s="137">
+      <c r="D40" s="136">
         <v>-0.93883069804431063</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="137">
+      <c r="A41" s="136">
         <v>16</v>
       </c>
-      <c r="B41" s="137">
+      <c r="B41" s="136">
         <v>16.266071428571429</v>
       </c>
-      <c r="C41" s="137">
+      <c r="C41" s="136">
         <v>-0.76607142857142918</v>
       </c>
-      <c r="D41" s="137">
+      <c r="D41" s="136">
         <v>-1.2469299364117945</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="137">
+      <c r="A42" s="136">
         <v>17</v>
       </c>
-      <c r="B42" s="137">
+      <c r="B42" s="136">
         <v>17.955357142857146</v>
       </c>
-      <c r="C42" s="137">
+      <c r="C42" s="136">
         <v>-0.4553571428571459</v>
       </c>
-      <c r="D42" s="137">
+      <c r="D42" s="136">
         <v>-0.74118213003498712</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="137">
+      <c r="A43" s="136">
         <v>18</v>
       </c>
-      <c r="B43" s="137">
+      <c r="B43" s="136">
         <v>19.644642857142859</v>
       </c>
-      <c r="C43" s="137">
+      <c r="C43" s="136">
         <v>-0.14464285714285907</v>
       </c>
-      <c r="D43" s="137">
+      <c r="D43" s="136">
         <v>-0.23543432365817393</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="137">
+      <c r="A44" s="136">
         <v>19</v>
       </c>
-      <c r="B44" s="137">
+      <c r="B44" s="136">
         <v>17.736309523809524</v>
       </c>
-      <c r="C44" s="137">
+      <c r="C44" s="136">
         <v>-0.23630952380952408</v>
       </c>
-      <c r="D44" s="137">
+      <c r="D44" s="136">
         <v>-0.38463961519462514</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="137">
+      <c r="A45" s="136">
         <v>20</v>
       </c>
-      <c r="B45" s="137">
+      <c r="B45" s="136">
         <v>19.425595238095241</v>
       </c>
-      <c r="C45" s="137">
+      <c r="C45" s="136">
         <v>-0.4255952380952408</v>
       </c>
-      <c r="D45" s="137">
+      <c r="D45" s="136">
         <v>-0.69273885356211184</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="137">
+      <c r="A46" s="136">
         <v>21</v>
       </c>
-      <c r="B46" s="137">
+      <c r="B46" s="136">
         <v>21.114880952380954</v>
       </c>
-      <c r="C46" s="137">
+      <c r="C46" s="136">
         <v>-0.11488095238095397</v>
       </c>
-      <c r="D46" s="137">
+      <c r="D46" s="136">
         <v>-0.18699104718529874</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="137">
+      <c r="A47" s="136">
         <v>22</v>
       </c>
-      <c r="B47" s="137">
+      <c r="B47" s="136">
         <v>22.804166666666667</v>
       </c>
-      <c r="C47" s="137">
+      <c r="C47" s="136">
         <v>0.19583333333333286</v>
       </c>
-      <c r="D47" s="137">
+      <c r="D47" s="136">
         <v>0.31875675919151442</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="137">
+      <c r="A48" s="136">
         <v>23</v>
       </c>
-      <c r="B48" s="137">
+      <c r="B48" s="136">
         <v>24.493452380952384</v>
       </c>
-      <c r="C48" s="137">
+      <c r="C48" s="136">
         <v>0.50654761904761614</v>
       </c>
-      <c r="D48" s="137">
+      <c r="D48" s="136">
         <v>0.82450456556832175</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="138">
+      <c r="A49" s="137">
         <v>24</v>
       </c>
-      <c r="B49" s="138">
+      <c r="B49" s="137">
         <v>26.182738095238101</v>
       </c>
-      <c r="C49" s="138">
+      <c r="C49" s="137">
         <v>1.8172619047618994</v>
       </c>
-      <c r="D49" s="138">
+      <c r="D49" s="137">
         <v>2.9579464614337172</v>
       </c>
     </row>
@@ -15105,48 +15122,48 @@
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="140" t="s">
+      <c r="A3" s="139" t="s">
         <v>359</v>
       </c>
-      <c r="B3" s="140"/>
+      <c r="B3" s="139"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="137" t="s">
+      <c r="A4" s="136" t="s">
         <v>360</v>
       </c>
-      <c r="B4" s="137">
+      <c r="B4" s="136">
         <v>0.99923601209082613</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="136" t="s">
         <v>361</v>
       </c>
-      <c r="B5" s="137">
+      <c r="B5" s="136">
         <v>0.99847260785917769</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="137" t="s">
+      <c r="A6" s="136" t="s">
         <v>362</v>
       </c>
-      <c r="B6" s="142">
+      <c r="B6" s="141">
         <v>0.95294863548914033</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="137" t="s">
+      <c r="A7" s="136" t="s">
         <v>363</v>
       </c>
-      <c r="B7" s="137">
+      <c r="B7" s="136">
         <v>0.63937706804773409</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="138" t="s">
+      <c r="A8" s="137" t="s">
         <v>364</v>
       </c>
-      <c r="B8" s="138">
+      <c r="B8" s="137">
         <v>24</v>
       </c>
     </row>
@@ -15156,185 +15173,185 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="139"/>
-      <c r="B11" s="139" t="s">
+      <c r="A11" s="138"/>
+      <c r="B11" s="138" t="s">
         <v>369</v>
       </c>
-      <c r="C11" s="139" t="s">
+      <c r="C11" s="138" t="s">
         <v>370</v>
       </c>
-      <c r="D11" s="139" t="s">
+      <c r="D11" s="138" t="s">
         <v>371</v>
       </c>
-      <c r="E11" s="139" t="s">
+      <c r="E11" s="138" t="s">
         <v>372</v>
       </c>
-      <c r="F11" s="139" t="s">
+      <c r="F11" s="138" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="137" t="s">
+      <c r="A12" s="136" t="s">
         <v>366</v>
       </c>
-      <c r="B12" s="137">
+      <c r="B12" s="136">
         <v>2</v>
       </c>
-      <c r="C12" s="137">
+      <c r="C12" s="136">
         <v>5879.2563332268028</v>
       </c>
-      <c r="D12" s="137">
+      <c r="D12" s="136">
         <v>2939.6281666134014</v>
       </c>
-      <c r="E12" s="137">
+      <c r="E12" s="136">
         <v>7190.8178606561842</v>
       </c>
-      <c r="F12" s="137">
+      <c r="F12" s="136">
         <v>1.658295194250544E-30</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="137" t="s">
+      <c r="A13" s="136" t="s">
         <v>367</v>
       </c>
-      <c r="B13" s="137">
+      <c r="B13" s="136">
         <v>22</v>
       </c>
-      <c r="C13" s="137">
+      <c r="C13" s="136">
         <v>8.9936667731969688</v>
       </c>
-      <c r="D13" s="137">
+      <c r="D13" s="136">
         <v>0.40880303514531674</v>
       </c>
-      <c r="E13" s="137"/>
-      <c r="F13" s="137"/>
+      <c r="E13" s="136"/>
+      <c r="F13" s="136"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="138" t="s">
+      <c r="A14" s="137" t="s">
         <v>317</v>
       </c>
-      <c r="B14" s="138">
+      <c r="B14" s="137">
         <v>24</v>
       </c>
-      <c r="C14" s="138">
+      <c r="C14" s="137">
         <v>5888.25</v>
       </c>
-      <c r="D14" s="138"/>
-      <c r="E14" s="138"/>
-      <c r="F14" s="138"/>
+      <c r="D14" s="137"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="137"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="139"/>
-      <c r="B16" s="139" t="s">
+      <c r="A16" s="138"/>
+      <c r="B16" s="138" t="s">
         <v>374</v>
       </c>
-      <c r="C16" s="139" t="s">
+      <c r="C16" s="138" t="s">
         <v>363</v>
       </c>
-      <c r="D16" s="139" t="s">
+      <c r="D16" s="138" t="s">
         <v>375</v>
       </c>
-      <c r="E16" s="139" t="s">
+      <c r="E16" s="138" t="s">
         <v>376</v>
       </c>
-      <c r="F16" s="139" t="s">
+      <c r="F16" s="138" t="s">
         <v>377</v>
       </c>
-      <c r="G16" s="139" t="s">
+      <c r="G16" s="138" t="s">
         <v>378</v>
       </c>
-      <c r="H16" s="139" t="s">
+      <c r="H16" s="138" t="s">
         <v>379</v>
       </c>
-      <c r="I16" s="139" t="s">
+      <c r="I16" s="138" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="137" t="s">
+      <c r="A17" s="136" t="s">
         <v>368</v>
       </c>
-      <c r="B17" s="137">
+      <c r="B17" s="136">
         <v>0</v>
       </c>
-      <c r="C17" s="137" t="e">
+      <c r="C17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="D17" s="137" t="e">
+      <c r="D17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E17" s="137" t="e">
+      <c r="E17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="F17" s="137" t="e">
+      <c r="F17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="G17" s="137" t="e">
+      <c r="G17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="H17" s="137" t="e">
+      <c r="H17" s="136" t="e">
         <v>#N/A</v>
       </c>
-      <c r="I17" s="137" t="e">
+      <c r="I17" s="136" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="137" t="s">
+      <c r="A18" s="136" t="s">
         <v>349</v>
       </c>
-      <c r="B18" s="137">
+      <c r="B18" s="136">
         <v>0.1629082774049217</v>
       </c>
-      <c r="C18" s="137">
+      <c r="C18" s="136">
         <v>3.3127900815938349E-3</v>
       </c>
-      <c r="D18" s="137">
+      <c r="D18" s="136">
         <v>49.175550938181992</v>
       </c>
-      <c r="E18" s="137">
+      <c r="E18" s="136">
         <v>5.4013091173267767E-24</v>
       </c>
-      <c r="F18" s="137">
+      <c r="F18" s="136">
         <v>0.15603797127508467</v>
       </c>
-      <c r="G18" s="137">
+      <c r="G18" s="136">
         <v>0.16977858353475872</v>
       </c>
-      <c r="H18" s="137">
+      <c r="H18" s="136">
         <v>0.15603797127508467</v>
       </c>
-      <c r="I18" s="137">
+      <c r="I18" s="136">
         <v>0.16977858353475872</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="138" t="s">
+      <c r="A19" s="137" t="s">
         <v>356</v>
       </c>
-      <c r="B19" s="138">
+      <c r="B19" s="137">
         <v>1.2974027910940667E-2</v>
       </c>
-      <c r="C19" s="138">
+      <c r="C19" s="137">
         <v>3.330620646154739E-4</v>
       </c>
-      <c r="D19" s="138">
+      <c r="D19" s="137">
         <v>38.953784562404053</v>
       </c>
-      <c r="E19" s="138">
+      <c r="E19" s="137">
         <v>8.5990489859870578E-22</v>
       </c>
-      <c r="F19" s="138">
+      <c r="F19" s="137">
         <v>1.2283299465194126E-2</v>
       </c>
-      <c r="G19" s="138">
+      <c r="G19" s="137">
         <v>1.3664756356687209E-2</v>
       </c>
-      <c r="H19" s="138">
+      <c r="H19" s="137">
         <v>1.2283299465194126E-2</v>
       </c>
-      <c r="I19" s="138">
+      <c r="I19" s="137">
         <v>1.3664756356687209E-2</v>
       </c>
     </row>
@@ -15345,352 +15362,352 @@
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="139" t="s">
+      <c r="A25" s="138" t="s">
         <v>382</v>
       </c>
-      <c r="B25" s="139" t="s">
+      <c r="B25" s="138" t="s">
         <v>383</v>
       </c>
-      <c r="C25" s="139" t="s">
+      <c r="C25" s="138" t="s">
         <v>384</v>
       </c>
-      <c r="D25" s="139" t="s">
+      <c r="D25" s="138" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="137">
+      <c r="A26" s="136">
         <v>1</v>
       </c>
-      <c r="B26" s="137">
+      <c r="B26" s="136">
         <v>4.8872483221476513</v>
       </c>
-      <c r="C26" s="137">
+      <c r="C26" s="136">
         <v>1.1127516778523487</v>
       </c>
-      <c r="D26" s="137">
+      <c r="D26" s="136">
         <v>1.8177555632337312</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="137">
+      <c r="A27" s="136">
         <v>2</v>
       </c>
-      <c r="B27" s="137">
+      <c r="B27" s="136">
         <v>6.5163310961968683</v>
       </c>
-      <c r="C27" s="137">
+      <c r="C27" s="136">
         <v>0.48366890380313166</v>
       </c>
-      <c r="D27" s="137">
+      <c r="D27" s="136">
         <v>0.79010605703886705</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="137">
+      <c r="A28" s="136">
         <v>3</v>
       </c>
-      <c r="B28" s="137">
+      <c r="B28" s="136">
         <v>8.1454138702460845</v>
       </c>
-      <c r="C28" s="137">
+      <c r="C28" s="136">
         <v>0.35458612975391546</v>
       </c>
-      <c r="D28" s="137">
+      <c r="D28" s="136">
         <v>0.57924056448039174</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="137">
+      <c r="A29" s="136">
         <v>4</v>
       </c>
-      <c r="B29" s="137">
+      <c r="B29" s="136">
         <v>9.7744966442953025</v>
       </c>
-      <c r="C29" s="137">
+      <c r="C29" s="136">
         <v>0.22550335570469748</v>
       </c>
-      <c r="D29" s="137">
+      <c r="D29" s="136">
         <v>0.36837507192191343</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="137">
+      <c r="A30" s="136">
         <v>5</v>
       </c>
-      <c r="B30" s="137">
+      <c r="B30" s="136">
         <v>11.403579418344519</v>
       </c>
-      <c r="C30" s="137">
+      <c r="C30" s="136">
         <v>9.6420581655481286E-2</v>
       </c>
-      <c r="D30" s="137">
+      <c r="D30" s="136">
         <v>0.15750957936343804</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="137">
+      <c r="A31" s="136">
         <v>6</v>
       </c>
-      <c r="B31" s="137">
+      <c r="B31" s="136">
         <v>13.032662192393737</v>
       </c>
-      <c r="C31" s="137">
+      <c r="C31" s="136">
         <v>-3.2662192393736689E-2</v>
       </c>
-      <c r="D31" s="137">
+      <c r="D31" s="136">
         <v>-5.335591319504026E-2</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="137">
+      <c r="A32" s="136">
         <v>7</v>
       </c>
-      <c r="B32" s="137">
+      <c r="B32" s="136">
         <v>8.1307552998828179</v>
       </c>
-      <c r="C32" s="137">
+      <c r="C32" s="136">
         <v>-0.13075529988281787</v>
       </c>
-      <c r="D32" s="137">
+      <c r="D32" s="136">
         <v>-0.21359767728503481</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="137">
+      <c r="A33" s="136">
         <v>8</v>
       </c>
-      <c r="B33" s="137">
+      <c r="B33" s="136">
         <v>9.7598380739320358</v>
       </c>
-      <c r="C33" s="137">
+      <c r="C33" s="136">
         <v>-0.25983807393203584</v>
       </c>
-      <c r="D33" s="137">
+      <c r="D33" s="136">
         <v>-0.42446316984351312</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="137">
+      <c r="A34" s="136">
         <v>9</v>
       </c>
-      <c r="B34" s="137">
+      <c r="B34" s="136">
         <v>11.388920847981252</v>
       </c>
-      <c r="C34" s="137">
+      <c r="C34" s="136">
         <v>-0.38892084798125204</v>
       </c>
-      <c r="D34" s="137">
+      <c r="D34" s="136">
         <v>-0.63532866240198849</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="137">
+      <c r="A35" s="136">
         <v>10</v>
       </c>
-      <c r="B35" s="137">
+      <c r="B35" s="136">
         <v>13.01800362203047</v>
       </c>
-      <c r="C35" s="137">
+      <c r="C35" s="136">
         <v>-0.51800362203047001</v>
       </c>
-      <c r="D35" s="137">
+      <c r="D35" s="136">
         <v>-0.84619415496046679</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="137">
+      <c r="A36" s="136">
         <v>11</v>
       </c>
-      <c r="B36" s="137">
+      <c r="B36" s="136">
         <v>14.647086396079686</v>
       </c>
-      <c r="C36" s="137">
+      <c r="C36" s="136">
         <v>-0.64708639607968621</v>
       </c>
-      <c r="D36" s="137">
+      <c r="D36" s="136">
         <v>-1.0570596475189422</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="137">
+      <c r="A37" s="136">
         <v>12</v>
       </c>
-      <c r="B37" s="137">
+      <c r="B37" s="136">
         <v>16.276169170128902</v>
       </c>
-      <c r="C37" s="137">
+      <c r="C37" s="136">
         <v>-0.27616917012890241</v>
       </c>
-      <c r="D37" s="137">
+      <c r="D37" s="136">
         <v>-0.45114112644103033</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="137">
+      <c r="A38" s="136">
         <v>13</v>
       </c>
-      <c r="B38" s="137">
+      <c r="B38" s="136">
         <v>11.374262277617985</v>
       </c>
-      <c r="C38" s="137">
+      <c r="C38" s="136">
         <v>-0.37426227761798536</v>
       </c>
-      <c r="D38" s="137">
+      <c r="D38" s="136">
         <v>-0.61138289053102779</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="137">
+      <c r="A39" s="136">
         <v>14</v>
       </c>
-      <c r="B39" s="137">
+      <c r="B39" s="136">
         <v>13.003345051667203</v>
       </c>
-      <c r="C39" s="137">
+      <c r="C39" s="136">
         <v>-0.50334505166720334</v>
       </c>
-      <c r="D39" s="137">
+      <c r="D39" s="136">
         <v>-0.8222483830895061</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="137">
+      <c r="A40" s="136">
         <v>15</v>
       </c>
-      <c r="B40" s="137">
+      <c r="B40" s="136">
         <v>14.63242782571642</v>
       </c>
-      <c r="C40" s="137">
+      <c r="C40" s="136">
         <v>-0.63242782571641953</v>
       </c>
-      <c r="D40" s="137">
+      <c r="D40" s="136">
         <v>-1.0331138756479814</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="137">
+      <c r="A41" s="136">
         <v>16</v>
       </c>
-      <c r="B41" s="137">
+      <c r="B41" s="136">
         <v>16.261510599765636</v>
       </c>
-      <c r="C41" s="137">
+      <c r="C41" s="136">
         <v>-0.76151059976563573</v>
       </c>
-      <c r="D41" s="137">
+      <c r="D41" s="136">
         <v>-1.2439793682064568</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="137">
+      <c r="A42" s="136">
         <v>17</v>
       </c>
-      <c r="B42" s="137">
+      <c r="B42" s="136">
         <v>17.890593373814852</v>
       </c>
-      <c r="C42" s="137">
+      <c r="C42" s="136">
         <v>-0.39059337381485193</v>
       </c>
-      <c r="D42" s="137">
+      <c r="D42" s="136">
         <v>-0.63806084712854505</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="137">
+      <c r="A43" s="136">
         <v>18</v>
       </c>
-      <c r="B43" s="137">
+      <c r="B43" s="136">
         <v>19.519676147864072</v>
       </c>
-      <c r="C43" s="137">
+      <c r="C43" s="136">
         <v>-1.967614786407168E-2</v>
       </c>
-      <c r="D43" s="137">
+      <c r="D43" s="136">
         <v>-3.2142326050638992E-2</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="137">
+      <c r="A44" s="136">
         <v>19</v>
       </c>
-      <c r="B44" s="137">
+      <c r="B44" s="136">
         <v>17.861276233088319</v>
       </c>
-      <c r="C44" s="137">
+      <c r="C44" s="136">
         <v>-0.36127623308831858</v>
       </c>
-      <c r="D44" s="137">
+      <c r="D44" s="136">
         <v>-0.59016930338662366</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="137">
+      <c r="A45" s="136">
         <v>20</v>
       </c>
-      <c r="B45" s="137">
+      <c r="B45" s="136">
         <v>19.490359007137535</v>
       </c>
-      <c r="C45" s="137">
+      <c r="C45" s="136">
         <v>-0.49035900713753477</v>
       </c>
-      <c r="D45" s="137">
+      <c r="D45" s="136">
         <v>-0.80103479594509897</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="137">
+      <c r="A46" s="136">
         <v>21</v>
       </c>
-      <c r="B46" s="137">
+      <c r="B46" s="136">
         <v>21.119441781186751</v>
       </c>
-      <c r="C46" s="137">
+      <c r="C46" s="136">
         <v>-0.11944178118675097</v>
       </c>
-      <c r="D46" s="137">
+      <c r="D46" s="136">
         <v>-0.19511627486718716</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="137">
+      <c r="A47" s="136">
         <v>22</v>
       </c>
-      <c r="B47" s="137">
+      <c r="B47" s="136">
         <v>22.748524555235971</v>
       </c>
-      <c r="C47" s="137">
+      <c r="C47" s="136">
         <v>0.25147544476402928</v>
       </c>
-      <c r="D47" s="137">
+      <c r="D47" s="136">
         <v>0.41080224621071887</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="137">
+      <c r="A48" s="136">
         <v>23</v>
       </c>
-      <c r="B48" s="137">
+      <c r="B48" s="136">
         <v>24.377607329285187</v>
       </c>
-      <c r="C48" s="137">
+      <c r="C48" s="136">
         <v>0.62239267071481308</v>
       </c>
-      <c r="D48" s="137">
+      <c r="D48" s="136">
         <v>1.0167207672886307</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="138">
+      <c r="A49" s="137">
         <v>24</v>
       </c>
-      <c r="B49" s="138">
+      <c r="B49" s="137">
         <v>26.006690103334407</v>
       </c>
-      <c r="C49" s="138">
+      <c r="C49" s="137">
         <v>1.9933098966655933</v>
       </c>
-      <c r="D49" s="138">
+      <c r="D49" s="137">
         <v>3.2562073156393114</v>
       </c>
     </row>
@@ -15705,7 +15722,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:L184"/>
+  <dimension ref="A1:L201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -15964,7 +15981,7 @@
       <c r="H12" t="s">
         <v>44</v>
       </c>
-      <c r="I12" s="112">
+      <c r="I12" s="111">
         <v>0</v>
       </c>
       <c r="J12" t="s">
@@ -15981,7 +15998,7 @@
       <c r="H13" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="158">
+      <c r="I13" s="157">
         <v>0</v>
       </c>
       <c r="J13" t="s">
@@ -15995,7 +16012,7 @@
       <c r="H14" t="s">
         <v>47</v>
       </c>
-      <c r="I14" s="158">
+      <c r="I14" s="157">
         <v>0</v>
       </c>
       <c r="J14" t="s">
@@ -16470,13 +16487,13 @@
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
-      <c r="D46" s="111" t="s">
+      <c r="D46" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="E46" s="111"/>
-      <c r="F46" s="111"/>
-      <c r="G46" s="111"/>
-      <c r="H46" s="111" t="s">
+      <c r="E46" s="110"/>
+      <c r="F46" s="110"/>
+      <c r="G46" s="110"/>
+      <c r="H46" s="110" t="s">
         <v>301</v>
       </c>
       <c r="I46" s="2">
@@ -16486,7 +16503,7 @@
       <c r="J46" t="s">
         <v>134</v>
       </c>
-      <c r="K46" s="110" t="s">
+      <c r="K46" s="109" t="s">
         <v>334</v>
       </c>
       <c r="L46" t="s">
@@ -16497,13 +16514,13 @@
       <c r="A47" t="s">
         <v>2</v>
       </c>
-      <c r="D47" s="111" t="s">
+      <c r="D47" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E47" s="111"/>
-      <c r="F47" s="111"/>
-      <c r="G47" s="111"/>
-      <c r="H47" s="111" t="s">
+      <c r="E47" s="110"/>
+      <c r="F47" s="110"/>
+      <c r="G47" s="110"/>
+      <c r="H47" s="110" t="s">
         <v>344</v>
       </c>
       <c r="I47" s="93">
@@ -16520,16 +16537,16 @@
       <c r="A48" t="s">
         <v>2</v>
       </c>
-      <c r="D48" s="111" t="s">
+      <c r="D48" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="111"/>
-      <c r="F48" s="111"/>
-      <c r="G48" s="111"/>
-      <c r="H48" s="111" t="s">
+      <c r="E48" s="110"/>
+      <c r="F48" s="110"/>
+      <c r="G48" s="110"/>
+      <c r="H48" s="110" t="s">
         <v>389</v>
       </c>
-      <c r="I48" s="112">
+      <c r="I48" s="111">
         <f>I47+(I95/0.5-I47)/(I90*30.4)*I29</f>
         <v>130.26609162869005</v>
       </c>
@@ -16544,16 +16561,16 @@
       <c r="A49" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="111" t="s">
+      <c r="D49" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E49" s="111"/>
-      <c r="F49" s="111"/>
-      <c r="G49" s="111"/>
-      <c r="H49" s="111" t="s">
+      <c r="E49" s="110"/>
+      <c r="F49" s="110"/>
+      <c r="G49" s="110"/>
+      <c r="H49" s="110" t="s">
         <v>330</v>
       </c>
-      <c r="I49" s="112">
+      <c r="I49" s="111">
         <f>I$50</f>
         <v>339.02685500000001</v>
       </c>
@@ -16568,13 +16585,13 @@
       <c r="A50" t="s">
         <v>2</v>
       </c>
-      <c r="D50" s="111" t="s">
+      <c r="D50" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E50" s="111"/>
-      <c r="F50" s="111"/>
-      <c r="G50" s="111"/>
-      <c r="H50" s="111" t="s">
+      <c r="E50" s="110"/>
+      <c r="F50" s="110"/>
+      <c r="G50" s="110"/>
+      <c r="H50" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I50" s="2">
@@ -16584,7 +16601,7 @@
       <c r="J50" t="s">
         <v>134</v>
       </c>
-      <c r="K50" s="110" t="s">
+      <c r="K50" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L50" t="s">
@@ -16595,13 +16612,13 @@
       <c r="A51" t="s">
         <v>2</v>
       </c>
-      <c r="D51" s="111" t="s">
+      <c r="D51" s="110" t="s">
         <v>33</v>
       </c>
-      <c r="E51" s="111"/>
-      <c r="F51" s="111"/>
-      <c r="G51" s="111"/>
-      <c r="H51" s="111" t="s">
+      <c r="E51" s="110"/>
+      <c r="F51" s="110"/>
+      <c r="G51" s="110"/>
+      <c r="H51" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I51" s="2">
@@ -16611,7 +16628,7 @@
       <c r="J51" t="s">
         <v>134</v>
       </c>
-      <c r="K51" s="110" t="s">
+      <c r="K51" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L51" t="s">
@@ -16622,13 +16639,13 @@
       <c r="A52" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="111" t="s">
+      <c r="D52" s="110" t="s">
         <v>34</v>
       </c>
-      <c r="E52" s="111"/>
-      <c r="F52" s="111"/>
-      <c r="G52" s="111"/>
-      <c r="H52" s="111" t="s">
+      <c r="E52" s="110"/>
+      <c r="F52" s="110"/>
+      <c r="G52" s="110"/>
+      <c r="H52" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I52" s="2">
@@ -16638,7 +16655,7 @@
       <c r="J52" t="s">
         <v>134</v>
       </c>
-      <c r="K52" s="110" t="s">
+      <c r="K52" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L52" t="s">
@@ -16649,13 +16666,13 @@
       <c r="A53" t="s">
         <v>2</v>
       </c>
-      <c r="D53" s="111" t="s">
+      <c r="D53" s="110" t="s">
         <v>35</v>
       </c>
-      <c r="E53" s="111"/>
-      <c r="F53" s="111"/>
-      <c r="G53" s="111"/>
-      <c r="H53" s="111" t="s">
+      <c r="E53" s="110"/>
+      <c r="F53" s="110"/>
+      <c r="G53" s="110"/>
+      <c r="H53" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I53" s="2">
@@ -16665,7 +16682,7 @@
       <c r="J53" t="s">
         <v>134</v>
       </c>
-      <c r="K53" s="110" t="s">
+      <c r="K53" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L53" t="s">
@@ -16694,13 +16711,13 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
-      <c r="D55" s="111" t="s">
+      <c r="D55" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="E55" s="111"/>
-      <c r="F55" s="111"/>
-      <c r="G55" s="111"/>
-      <c r="H55" s="111" t="s">
+      <c r="E55" s="110"/>
+      <c r="F55" s="110"/>
+      <c r="G55" s="110"/>
+      <c r="H55" s="110" t="s">
         <v>301</v>
       </c>
       <c r="I55" s="2">
@@ -16710,7 +16727,7 @@
       <c r="J55" t="s">
         <v>134</v>
       </c>
-      <c r="K55" s="110" t="s">
+      <c r="K55" s="109" t="s">
         <v>334</v>
       </c>
       <c r="L55" t="s">
@@ -16721,13 +16738,13 @@
       <c r="A56" t="s">
         <v>39</v>
       </c>
-      <c r="D56" s="111" t="s">
+      <c r="D56" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E56" s="111"/>
-      <c r="F56" s="111"/>
-      <c r="G56" s="111"/>
-      <c r="H56" s="111" t="s">
+      <c r="E56" s="110"/>
+      <c r="F56" s="110"/>
+      <c r="G56" s="110"/>
+      <c r="H56" s="110" t="s">
         <v>344</v>
       </c>
       <c r="I56" s="93">
@@ -16744,16 +16761,16 @@
       <c r="A57" t="s">
         <v>39</v>
       </c>
-      <c r="D57" s="111" t="s">
+      <c r="D57" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E57" s="111"/>
-      <c r="F57" s="111"/>
-      <c r="G57" s="111"/>
-      <c r="H57" s="111" t="s">
+      <c r="E57" s="110"/>
+      <c r="F57" s="110"/>
+      <c r="G57" s="110"/>
+      <c r="H57" s="110" t="s">
         <v>389</v>
       </c>
-      <c r="I57" s="112">
+      <c r="I57" s="111">
         <f>I56+(I115/0.5-I56)/(I110*30.4)*I40</f>
         <v>215.80423925763492</v>
       </c>
@@ -16768,16 +16785,16 @@
       <c r="A58" t="s">
         <v>39</v>
       </c>
-      <c r="D58" s="111" t="s">
+      <c r="D58" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E58" s="111"/>
-      <c r="F58" s="111"/>
-      <c r="G58" s="111"/>
-      <c r="H58" s="111" t="s">
+      <c r="E58" s="110"/>
+      <c r="F58" s="110"/>
+      <c r="G58" s="110"/>
+      <c r="H58" s="110" t="s">
         <v>330</v>
       </c>
-      <c r="I58" s="112">
+      <c r="I58" s="111">
         <f>I$59</f>
         <v>314.63230679999998</v>
       </c>
@@ -16792,13 +16809,13 @@
       <c r="A59" t="s">
         <v>39</v>
       </c>
-      <c r="D59" s="111" t="s">
+      <c r="D59" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="E59" s="111"/>
-      <c r="F59" s="111"/>
-      <c r="G59" s="111"/>
-      <c r="H59" s="111" t="s">
+      <c r="E59" s="110"/>
+      <c r="F59" s="110"/>
+      <c r="G59" s="110"/>
+      <c r="H59" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I59" s="2">
@@ -16808,7 +16825,7 @@
       <c r="J59" t="s">
         <v>134</v>
       </c>
-      <c r="K59" s="110" t="s">
+      <c r="K59" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L59" t="s">
@@ -16819,13 +16836,13 @@
       <c r="A60" t="s">
         <v>39</v>
       </c>
-      <c r="D60" s="111" t="s">
+      <c r="D60" s="110" t="s">
         <v>33</v>
       </c>
-      <c r="E60" s="111"/>
-      <c r="F60" s="111"/>
-      <c r="G60" s="111"/>
-      <c r="H60" s="111" t="s">
+      <c r="E60" s="110"/>
+      <c r="F60" s="110"/>
+      <c r="G60" s="110"/>
+      <c r="H60" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I60" s="2">
@@ -16835,7 +16852,7 @@
       <c r="J60" t="s">
         <v>134</v>
       </c>
-      <c r="K60" s="110" t="s">
+      <c r="K60" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L60" t="s">
@@ -16846,13 +16863,13 @@
       <c r="A61" t="s">
         <v>39</v>
       </c>
-      <c r="D61" s="111" t="s">
+      <c r="D61" s="110" t="s">
         <v>34</v>
       </c>
-      <c r="E61" s="111"/>
-      <c r="F61" s="111"/>
-      <c r="G61" s="111"/>
-      <c r="H61" s="111" t="s">
+      <c r="E61" s="110"/>
+      <c r="F61" s="110"/>
+      <c r="G61" s="110"/>
+      <c r="H61" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I61" s="2">
@@ -16862,7 +16879,7 @@
       <c r="J61" t="s">
         <v>134</v>
       </c>
-      <c r="K61" s="110" t="s">
+      <c r="K61" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L61" t="s">
@@ -16873,13 +16890,13 @@
       <c r="A62" t="s">
         <v>39</v>
       </c>
-      <c r="D62" s="111" t="s">
+      <c r="D62" s="110" t="s">
         <v>35</v>
       </c>
-      <c r="E62" s="111"/>
-      <c r="F62" s="111"/>
-      <c r="G62" s="111"/>
-      <c r="H62" s="111" t="s">
+      <c r="E62" s="110"/>
+      <c r="F62" s="110"/>
+      <c r="G62" s="110"/>
+      <c r="H62" s="110" t="s">
         <v>297</v>
       </c>
       <c r="I62" s="2">
@@ -16889,7 +16906,7 @@
       <c r="J62" t="s">
         <v>134</v>
       </c>
-      <c r="K62" s="110" t="s">
+      <c r="K62" s="109" t="s">
         <v>332</v>
       </c>
       <c r="L62" t="s">
@@ -17539,7 +17556,7 @@
       <c r="H99" t="s">
         <v>36</v>
       </c>
-      <c r="I99" s="159">
+      <c r="I99" s="158">
         <v>0</v>
       </c>
       <c r="J99" s="93" t="s">
@@ -17926,7 +17943,7 @@
       <c r="H119" t="s">
         <v>36</v>
       </c>
-      <c r="I119" s="159">
+      <c r="I119" s="158">
         <v>0</v>
       </c>
       <c r="J119" s="93" t="s">
@@ -18877,163 +18894,398 @@
       </c>
     </row>
     <row r="176" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H176" s="93" t="s">
+      <c r="H176" s="160" t="s">
         <v>327</v>
       </c>
-      <c r="I176" s="93">
+      <c r="I176" s="160">
         <v>0</v>
       </c>
-      <c r="J176" s="93" t="s">
+      <c r="J176" s="160" t="s">
         <v>328</v>
       </c>
-      <c r="K176" s="93" t="s">
+      <c r="K176" s="160" t="s">
         <v>430</v>
       </c>
     </row>
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H177" s="93"/>
+      <c r="I177" s="93"/>
+      <c r="J177" s="93"/>
+      <c r="K177" s="93"/>
+    </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A178" s="102" t="s">
+      <c r="A178" s="94" t="s">
+        <v>432</v>
+      </c>
+      <c r="B178" s="94"/>
+      <c r="C178" s="94"/>
+      <c r="D178" s="95"/>
+      <c r="E178" s="95"/>
+      <c r="F178" s="95"/>
+      <c r="G178" s="95"/>
+      <c r="H178" s="95"/>
+      <c r="I178" s="95"/>
+      <c r="J178" s="95" t="s">
+        <v>9</v>
+      </c>
+      <c r="K178" s="95" t="s">
+        <v>434</v>
+      </c>
+      <c r="L178" s="95"/>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A179" s="97" t="s">
+        <v>304</v>
+      </c>
+      <c r="B179" s="97"/>
+      <c r="C179" s="97"/>
+      <c r="D179" s="98"/>
+      <c r="E179" s="98"/>
+      <c r="F179" s="98"/>
+      <c r="G179" s="98"/>
+      <c r="H179" s="98"/>
+      <c r="I179" s="99"/>
+      <c r="J179" s="98"/>
+      <c r="K179" s="98"/>
+      <c r="L179" s="98"/>
+    </row>
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>2</v>
+      </c>
+      <c r="D180" t="s">
+        <v>18</v>
+      </c>
+      <c r="H180" t="s">
+        <v>433</v>
+      </c>
+      <c r="J180" s="93">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>2</v>
+      </c>
+      <c r="D181" t="s">
+        <v>20</v>
+      </c>
+      <c r="H181" t="s">
+        <v>433</v>
+      </c>
+      <c r="J181" s="93">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>2</v>
+      </c>
+      <c r="D182" t="s">
+        <v>35</v>
+      </c>
+      <c r="H182" t="s">
+        <v>433</v>
+      </c>
+      <c r="J182" s="93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>2</v>
+      </c>
+      <c r="D183" t="s">
+        <v>33</v>
+      </c>
+      <c r="H183" t="s">
+        <v>433</v>
+      </c>
+      <c r="J183" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>2</v>
+      </c>
+      <c r="D184" t="s">
+        <v>34</v>
+      </c>
+      <c r="H184" t="s">
+        <v>433</v>
+      </c>
+      <c r="J184" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>2</v>
+      </c>
+      <c r="D185" t="s">
+        <v>431</v>
+      </c>
+      <c r="H185" t="s">
+        <v>433</v>
+      </c>
+      <c r="J185" s="93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A187" s="100" t="s">
+        <v>305</v>
+      </c>
+      <c r="B187" s="100"/>
+      <c r="C187" s="100"/>
+      <c r="D187" s="101"/>
+      <c r="E187" s="101"/>
+      <c r="F187" s="101"/>
+      <c r="G187" s="101"/>
+      <c r="H187" s="101"/>
+      <c r="I187" s="101"/>
+      <c r="J187" s="101"/>
+      <c r="K187" s="101"/>
+      <c r="L187" s="101"/>
+    </row>
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>39</v>
+      </c>
+      <c r="D188" t="s">
+        <v>18</v>
+      </c>
+      <c r="H188" t="s">
+        <v>433</v>
+      </c>
+      <c r="J188" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>39</v>
+      </c>
+      <c r="D189" t="s">
+        <v>20</v>
+      </c>
+      <c r="H189" t="s">
+        <v>433</v>
+      </c>
+      <c r="J189" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>39</v>
+      </c>
+      <c r="D190" t="s">
+        <v>35</v>
+      </c>
+      <c r="H190" t="s">
+        <v>433</v>
+      </c>
+      <c r="J190" s="93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>39</v>
+      </c>
+      <c r="D191" t="s">
+        <v>33</v>
+      </c>
+      <c r="H191" t="s">
+        <v>433</v>
+      </c>
+      <c r="J191" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>39</v>
+      </c>
+      <c r="D192" t="s">
+        <v>34</v>
+      </c>
+      <c r="H192" t="s">
+        <v>433</v>
+      </c>
+      <c r="J192" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>39</v>
+      </c>
+      <c r="D193" t="s">
+        <v>431</v>
+      </c>
+      <c r="H193" t="s">
+        <v>433</v>
+      </c>
+      <c r="J193" s="93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A195" s="159" t="s">
         <v>306</v>
       </c>
-      <c r="B178" s="102"/>
-      <c r="C178" s="102"/>
-    </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A179" s="93" t="s">
+      <c r="B195" s="159"/>
+      <c r="C195" s="159"/>
+      <c r="D195" s="95"/>
+      <c r="E195" s="95"/>
+      <c r="F195" s="95"/>
+      <c r="G195" s="95"/>
+      <c r="H195" s="95"/>
+      <c r="I195" s="95"/>
+      <c r="J195" s="95"/>
+      <c r="K195" s="95"/>
+      <c r="L195" s="95"/>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A196" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D179" s="93" t="s">
+      <c r="D196" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="E179" s="93"/>
-      <c r="F179" s="93"/>
-      <c r="G179" s="93"/>
-      <c r="H179" s="93" t="s">
+      <c r="E196" s="93"/>
+      <c r="F196" s="93"/>
+      <c r="G196" s="93"/>
+      <c r="H196" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I179" s="93">
+      <c r="I196" s="93">
         <v>7.1</v>
       </c>
-      <c r="J179" s="93" t="s">
+      <c r="J196" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K179" s="93"/>
-      <c r="L179" s="93" t="s">
+      <c r="K196" s="93"/>
+      <c r="L196" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A180" s="93" t="s">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A197" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="D180" s="93" t="s">
+      <c r="D197" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="E180" s="93"/>
-      <c r="F180" s="93"/>
-      <c r="G180" s="93"/>
-      <c r="H180" s="93" t="s">
+      <c r="E197" s="93"/>
+      <c r="F197" s="93"/>
+      <c r="G197" s="93"/>
+      <c r="H197" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I180" s="93">
+      <c r="I197" s="93">
         <v>5.0999999999999996</v>
       </c>
-      <c r="J180" s="93" t="s">
+      <c r="J197" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K180" s="93"/>
-      <c r="L180" s="93" t="s">
+      <c r="K197" s="93"/>
+      <c r="L197" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A181" s="93"/>
-      <c r="D181" s="93" t="s">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A198" s="93"/>
+      <c r="D198" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="E181" s="93"/>
-      <c r="F181" s="93"/>
-      <c r="G181" s="93"/>
-      <c r="H181" s="93" t="s">
+      <c r="E198" s="93"/>
+      <c r="F198" s="93"/>
+      <c r="G198" s="93"/>
+      <c r="H198" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I181" s="93">
+      <c r="I198" s="93">
         <v>5.7</v>
       </c>
-      <c r="J181" s="93" t="s">
+      <c r="J198" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K181" s="93"/>
-      <c r="L181" s="93" t="s">
+      <c r="K198" s="93"/>
+      <c r="L198" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A182" s="93"/>
-      <c r="D182" s="93" t="s">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A199" s="93"/>
+      <c r="D199" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="E182" s="93"/>
-      <c r="F182" s="93"/>
-      <c r="G182" s="93"/>
-      <c r="H182" s="93" t="s">
+      <c r="E199" s="93"/>
+      <c r="F199" s="93"/>
+      <c r="G199" s="93"/>
+      <c r="H199" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I182" s="93">
+      <c r="I199" s="93">
         <v>7.7</v>
       </c>
-      <c r="J182" s="93" t="s">
+      <c r="J199" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K182" s="93"/>
-      <c r="L182" s="93" t="s">
+      <c r="K199" s="93"/>
+      <c r="L199" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A183" s="93"/>
-      <c r="D183" s="93" t="s">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A200" s="93"/>
+      <c r="D200" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="E183" s="93"/>
-      <c r="F183" s="93"/>
-      <c r="G183" s="93"/>
-      <c r="H183" s="93" t="s">
+      <c r="E200" s="93"/>
+      <c r="F200" s="93"/>
+      <c r="G200" s="93"/>
+      <c r="H200" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I183" s="93">
+      <c r="I200" s="93">
         <v>9.1</v>
       </c>
-      <c r="J183" s="93" t="s">
+      <c r="J200" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K183" s="93" t="s">
+      <c r="K200" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="L183" s="93" t="s">
+      <c r="L200" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A184" s="93"/>
-      <c r="D184" s="93" t="s">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A201" s="93"/>
+      <c r="D201" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E184" s="93"/>
-      <c r="F184" s="93"/>
-      <c r="G184" s="93"/>
-      <c r="H184" s="93" t="s">
+      <c r="E201" s="93"/>
+      <c r="F201" s="93"/>
+      <c r="G201" s="93"/>
+      <c r="H201" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I184" s="93">
+      <c r="I201" s="93">
         <v>9.1</v>
       </c>
-      <c r="J184" s="93" t="s">
+      <c r="J201" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K184" s="93" t="s">
+      <c r="K201" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="L184" s="93" t="s">
+      <c r="L201" s="93" t="s">
         <v>42</v>
       </c>
     </row>
@@ -21625,7 +21877,7 @@
       <c r="J40" s="15"/>
       <c r="K40" s="21"/>
       <c r="L40" s="22"/>
-      <c r="M40" s="104" t="s">
+      <c r="M40" s="103" t="s">
         <v>318</v>
       </c>
       <c r="N40" s="15"/>
@@ -21637,7 +21889,7 @@
       <c r="T40" s="15"/>
       <c r="U40" s="15"/>
       <c r="V40" s="15"/>
-      <c r="W40" s="107"/>
+      <c r="W40" s="106"/>
       <c r="X40" s="26"/>
       <c r="AA40" s="15"/>
       <c r="AB40" s="21"/>
@@ -21648,7 +21900,7 @@
       <c r="AG40" s="15"/>
       <c r="AH40" s="15"/>
       <c r="AI40" s="15"/>
-      <c r="AJ40" s="104" t="s">
+      <c r="AJ40" s="103" t="s">
         <v>318</v>
       </c>
       <c r="AK40" s="15"/>
@@ -21660,7 +21912,7 @@
       <c r="AQ40" s="15"/>
       <c r="AR40" s="15"/>
       <c r="AS40" s="15"/>
-      <c r="AT40" s="107"/>
+      <c r="AT40" s="106"/>
     </row>
     <row r="41" spans="2:46" x14ac:dyDescent="0.25">
       <c r="D41" s="12"/>
@@ -21668,7 +21920,7 @@
       <c r="J41" s="15"/>
       <c r="K41" s="21"/>
       <c r="L41" s="22"/>
-      <c r="M41" s="105" t="s">
+      <c r="M41" s="104" t="s">
         <v>319</v>
       </c>
       <c r="N41" s="15"/>
@@ -21677,7 +21929,7 @@
         <v>89</v>
       </c>
       <c r="Q41" s="15"/>
-      <c r="R41" s="109" t="s">
+      <c r="R41" s="108" t="s">
         <v>9</v>
       </c>
       <c r="S41" s="15"/>
@@ -21686,7 +21938,7 @@
       </c>
       <c r="U41" s="15"/>
       <c r="V41" s="15"/>
-      <c r="W41" s="107"/>
+      <c r="W41" s="106"/>
       <c r="X41" s="26"/>
       <c r="AA41" s="15"/>
       <c r="AB41" s="21"/>
@@ -21697,7 +21949,7 @@
       <c r="AG41" s="15"/>
       <c r="AH41" s="15"/>
       <c r="AI41" s="15"/>
-      <c r="AJ41" s="105" t="s">
+      <c r="AJ41" s="104" t="s">
         <v>319</v>
       </c>
       <c r="AK41" s="15"/>
@@ -21706,14 +21958,14 @@
         <v>14</v>
       </c>
       <c r="AN41" s="15"/>
-      <c r="AO41" s="109" t="s">
+      <c r="AO41" s="108" t="s">
         <v>9</v>
       </c>
       <c r="AP41" s="15"/>
       <c r="AQ41" s="15"/>
       <c r="AR41" s="15"/>
       <c r="AS41" s="15"/>
-      <c r="AT41" s="107"/>
+      <c r="AT41" s="106"/>
     </row>
     <row r="42" spans="2:46" x14ac:dyDescent="0.25">
       <c r="D42" s="12"/>
@@ -21721,7 +21973,7 @@
       <c r="J42" s="15"/>
       <c r="K42" s="21"/>
       <c r="L42" s="22"/>
-      <c r="M42" s="106" t="s">
+      <c r="M42" s="105" t="s">
         <v>320</v>
       </c>
       <c r="N42" s="47"/>
@@ -21739,7 +21991,7 @@
       </c>
       <c r="U42" s="47"/>
       <c r="V42" s="47"/>
-      <c r="W42" s="108"/>
+      <c r="W42" s="107"/>
       <c r="X42" s="26"/>
       <c r="AA42" s="15"/>
       <c r="AB42" s="21"/>
@@ -21750,7 +22002,7 @@
       <c r="AG42" s="15"/>
       <c r="AH42" s="15"/>
       <c r="AI42" s="15"/>
-      <c r="AJ42" s="106" t="s">
+      <c r="AJ42" s="105" t="s">
         <v>320</v>
       </c>
       <c r="AK42" s="47"/>
@@ -21766,7 +22018,7 @@
       <c r="AQ42" s="47"/>
       <c r="AR42" s="47"/>
       <c r="AS42" s="47"/>
-      <c r="AT42" s="108"/>
+      <c r="AT42" s="107"/>
     </row>
     <row r="43" spans="2:46" x14ac:dyDescent="0.25">
       <c r="D43" s="12"/>
@@ -21862,7 +22114,7 @@
         <f>SUM(D5:E5)</f>
         <v>316238</v>
       </c>
-      <c r="E46" s="103">
+      <c r="E46" s="102">
         <f>E5</f>
         <v>55025.411999999997</v>
       </c>
@@ -21908,7 +22160,7 @@
         <f>SUM(AA5:AB5)</f>
         <v>206514</v>
       </c>
-      <c r="E47" s="103">
+      <c r="E47" s="102">
         <f>AB5</f>
         <v>72692.928000000014</v>
       </c>
@@ -21954,7 +22206,7 @@
         <f>SUM(D9:E9,AA9:AB9)</f>
         <v>462203.76921728684</v>
       </c>
-      <c r="E48" s="103">
+      <c r="E48" s="102">
         <f>SUM(E9,AB9)</f>
         <v>85658.04919782767</v>
       </c>
@@ -22002,7 +22254,7 @@
         <f>SUM(D6:E8,AA6:AB8)</f>
         <v>491678.55122292211</v>
       </c>
-      <c r="E49" s="103">
+      <c r="E49" s="102">
         <f>SUM(E6:E8,AB6:AB8)</f>
         <v>97115.906082827161</v>
       </c>
@@ -22096,7 +22348,7 @@
         <f>SUM(F5:G5,AC5:AD5)</f>
         <v>143608.72911893675</v>
       </c>
-      <c r="E50" s="103">
+      <c r="E50" s="102">
         <f>SUM(G5,AD5)</f>
         <v>33025.146960105732</v>
       </c>
@@ -22215,7 +22467,7 @@
         <f>SUM(F6:G6,AC6:AD6)</f>
         <v>56446.350672823188</v>
       </c>
-      <c r="E51" s="103">
+      <c r="E51" s="102">
         <f>SUM(G6,AD6)</f>
         <v>13122.812032834503</v>
       </c>
@@ -22334,7 +22586,7 @@
         <f>SUM(F7:G7,AC7:AD7)</f>
         <v>35750.513487991702</v>
       </c>
-      <c r="E52" s="103">
+      <c r="E52" s="102">
         <f>SUM(G7,AD7)</f>
         <v>11903.310295425101</v>
       </c>
@@ -22385,7 +22637,7 @@
         <f>SUM(F8:G8,AC8:AD8)</f>
         <v>183108.40482051656</v>
       </c>
-      <c r="E53" s="103">
+      <c r="E53" s="102">
         <f>SUM(G8,AD8)</f>
         <v>19474.403024226824</v>
       </c>
@@ -25121,7 +25373,7 @@
       </c>
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B105" s="156" t="s">
+      <c r="B105" s="155" t="s">
         <v>400</v>
       </c>
       <c r="C105" s="2">
@@ -25162,18 +25414,18 @@
       </c>
     </row>
     <row r="106" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="D106" s="156" t="s">
+      <c r="D106" s="155" t="s">
         <v>405</v>
       </c>
-      <c r="E106" s="157">
+      <c r="E106" s="156">
         <f>1/E105</f>
         <v>4.9969493593654671E-2</v>
       </c>
-      <c r="H106" s="157">
+      <c r="H106" s="156">
         <f>1/H105</f>
         <v>3.1568577532293592E-2</v>
       </c>
-      <c r="K106" s="157">
+      <c r="K106" s="156">
         <f>1/K105</f>
         <v>5.9876519298329253E-2</v>
       </c>
@@ -47026,16 +47278,16 @@
         <f>SUM(G4:I4)</f>
         <v>28</v>
       </c>
-      <c r="R4" s="141" t="s">
+      <c r="R4" s="140" t="s">
         <v>353</v>
       </c>
-      <c r="S4" s="119"/>
-      <c r="T4" s="119"/>
-      <c r="U4" s="119"/>
-      <c r="V4" s="119"/>
-      <c r="W4" s="119"/>
-      <c r="X4" s="113"/>
-      <c r="Y4" s="113"/>
+      <c r="S4" s="118"/>
+      <c r="T4" s="118"/>
+      <c r="U4" s="118"/>
+      <c r="V4" s="118"/>
+      <c r="W4" s="118"/>
+      <c r="X4" s="112"/>
+      <c r="Y4" s="112"/>
       <c r="AB4" t="s">
         <v>349</v>
       </c>
@@ -47082,29 +47334,29 @@
         <f t="shared" ref="N5:N7" si="0">SUM(G5:I5)</f>
         <v>37</v>
       </c>
-      <c r="R5" s="120" t="s">
+      <c r="R5" s="119" t="s">
         <v>355</v>
       </c>
-      <c r="S5" s="120" t="s">
+      <c r="S5" s="119" t="s">
         <v>354</v>
       </c>
-      <c r="T5" s="119"/>
-      <c r="U5" s="119"/>
-      <c r="V5" s="119"/>
-      <c r="W5" s="119"/>
-      <c r="X5" s="119"/>
-      <c r="Y5" s="119"/>
-      <c r="AB5" s="134">
+      <c r="T5" s="118"/>
+      <c r="U5" s="118"/>
+      <c r="V5" s="118"/>
+      <c r="W5" s="118"/>
+      <c r="X5" s="118"/>
+      <c r="Y5" s="118"/>
+      <c r="AB5" s="133">
         <v>30</v>
       </c>
-      <c r="AC5" s="134">
+      <c r="AC5" s="133">
         <f t="shared" ref="AC5:AC28" si="1">AB5^0.75</f>
         <v>12.818610191887021</v>
       </c>
-      <c r="AD5" s="134">
+      <c r="AD5" s="133">
         <v>0</v>
       </c>
-      <c r="AE5" s="126">
+      <c r="AE5" s="125">
         <v>6</v>
       </c>
     </row>
@@ -47141,35 +47393,35 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="R6" s="121" t="s">
+      <c r="R6" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="S6" s="122">
+      <c r="S6" s="121">
         <v>0</v>
       </c>
-      <c r="T6" s="123">
+      <c r="T6" s="122">
         <v>250</v>
       </c>
-      <c r="U6" s="123">
+      <c r="U6" s="122">
         <v>500</v>
       </c>
-      <c r="V6" s="124">
+      <c r="V6" s="123">
         <v>1000</v>
       </c>
-      <c r="W6" s="116"/>
-      <c r="X6" s="116"/>
-      <c r="Y6" s="116"/>
-      <c r="AB6" s="135">
+      <c r="W6" s="115"/>
+      <c r="X6" s="115"/>
+      <c r="Y6" s="115"/>
+      <c r="AB6" s="134">
         <v>40</v>
       </c>
-      <c r="AC6" s="135">
+      <c r="AC6" s="134">
         <f t="shared" si="1"/>
         <v>15.905414575341014</v>
       </c>
-      <c r="AD6" s="135">
+      <c r="AD6" s="134">
         <v>0</v>
       </c>
-      <c r="AE6" s="129">
+      <c r="AE6" s="128">
         <v>7</v>
       </c>
     </row>
@@ -47206,754 +47458,754 @@
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="R7" s="115">
+      <c r="R7" s="114">
         <v>30</v>
       </c>
-      <c r="S7" s="125">
+      <c r="S7" s="124">
         <v>6</v>
       </c>
-      <c r="T7" s="126">
+      <c r="T7" s="125">
         <v>8</v>
       </c>
-      <c r="U7" s="126">
+      <c r="U7" s="125">
         <v>11</v>
       </c>
-      <c r="V7" s="127">
+      <c r="V7" s="126">
         <v>17.5</v>
       </c>
-      <c r="W7" s="114"/>
-      <c r="X7" s="155" t="s">
+      <c r="W7" s="113"/>
+      <c r="X7" s="154" t="s">
         <v>390</v>
       </c>
-      <c r="Y7" s="114"/>
-      <c r="AB7" s="135">
+      <c r="Y7" s="113"/>
+      <c r="AB7" s="134">
         <v>50</v>
       </c>
-      <c r="AC7" s="135">
+      <c r="AC7" s="134">
         <f t="shared" si="1"/>
         <v>18.803015465431965</v>
       </c>
-      <c r="AD7" s="135">
+      <c r="AD7" s="134">
         <v>0</v>
       </c>
-      <c r="AE7" s="129">
+      <c r="AE7" s="128">
         <v>8.5</v>
       </c>
     </row>
     <row r="8" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R8" s="117">
+      <c r="R8" s="116">
         <v>40</v>
       </c>
-      <c r="S8" s="128">
+      <c r="S8" s="127">
         <v>7</v>
       </c>
-      <c r="T8" s="129">
+      <c r="T8" s="128">
         <v>9.5</v>
       </c>
-      <c r="U8" s="129">
+      <c r="U8" s="128">
         <v>12.5</v>
       </c>
-      <c r="V8" s="130">
+      <c r="V8" s="129">
         <v>19</v>
       </c>
-      <c r="W8" s="114"/>
+      <c r="W8" s="113"/>
       <c r="X8" t="s">
         <v>387</v>
       </c>
       <c r="Y8">
         <v>0</v>
       </c>
-      <c r="AB8" s="135">
+      <c r="AB8" s="134">
         <v>60</v>
       </c>
-      <c r="AC8" s="135">
+      <c r="AC8" s="134">
         <f t="shared" si="1"/>
         <v>21.558246717785043</v>
       </c>
-      <c r="AD8" s="135">
+      <c r="AD8" s="134">
         <v>0</v>
       </c>
-      <c r="AE8" s="129">
+      <c r="AE8" s="128">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R9" s="117">
+      <c r="R9" s="116">
         <v>50</v>
       </c>
-      <c r="S9" s="128">
+      <c r="S9" s="127">
         <v>8.5</v>
       </c>
-      <c r="T9" s="129">
+      <c r="T9" s="128">
         <v>11</v>
       </c>
-      <c r="U9" s="129">
+      <c r="U9" s="128">
         <v>14</v>
       </c>
-      <c r="V9" s="130">
+      <c r="V9" s="129">
         <v>21</v>
       </c>
-      <c r="W9" s="114"/>
+      <c r="W9" s="113"/>
       <c r="X9" t="s">
         <v>349</v>
       </c>
-      <c r="Y9" s="137">
+      <c r="Y9" s="136">
         <v>0.16</v>
       </c>
-      <c r="AB9" s="135">
+      <c r="AB9" s="134">
         <v>70</v>
       </c>
-      <c r="AC9" s="135">
+      <c r="AC9" s="134">
         <f t="shared" si="1"/>
         <v>24.200454924935883</v>
       </c>
-      <c r="AD9" s="135">
+      <c r="AD9" s="134">
         <v>0</v>
       </c>
-      <c r="AE9" s="129">
+      <c r="AE9" s="128">
         <v>11.5</v>
       </c>
     </row>
     <row r="10" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R10" s="117">
+      <c r="R10" s="116">
         <v>60</v>
       </c>
-      <c r="S10" s="128">
+      <c r="S10" s="127">
         <v>10</v>
       </c>
-      <c r="T10" s="129">
+      <c r="T10" s="128">
         <v>12.5</v>
       </c>
-      <c r="U10" s="129">
+      <c r="U10" s="128">
         <v>15.5</v>
       </c>
-      <c r="V10" s="130">
+      <c r="V10" s="129">
         <v>23</v>
       </c>
-      <c r="W10" s="114"/>
+      <c r="W10" s="113"/>
       <c r="X10" t="s">
         <v>356</v>
       </c>
       <c r="Y10">
         <v>12.5</v>
       </c>
-      <c r="AB10" s="136">
+      <c r="AB10" s="135">
         <v>80</v>
       </c>
-      <c r="AC10" s="136">
+      <c r="AC10" s="135">
         <f t="shared" si="1"/>
         <v>26.749612199056873</v>
       </c>
-      <c r="AD10" s="136">
+      <c r="AD10" s="135">
         <v>0</v>
       </c>
-      <c r="AE10" s="132">
+      <c r="AE10" s="131">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R11" s="117">
+      <c r="R11" s="116">
         <v>70</v>
       </c>
-      <c r="S11" s="128">
+      <c r="S11" s="127">
         <v>11.5</v>
       </c>
-      <c r="T11" s="129">
+      <c r="T11" s="128">
         <v>14</v>
       </c>
-      <c r="U11" s="129">
+      <c r="U11" s="128">
         <v>17.5</v>
       </c>
-      <c r="V11" s="130">
+      <c r="V11" s="129">
         <v>25</v>
       </c>
-      <c r="W11" s="116"/>
-      <c r="X11" s="116"/>
-      <c r="Y11" s="116"/>
-      <c r="AB11" s="134">
+      <c r="W11" s="115"/>
+      <c r="X11" s="115"/>
+      <c r="Y11" s="115"/>
+      <c r="AB11" s="133">
         <v>30</v>
       </c>
-      <c r="AC11" s="134">
+      <c r="AC11" s="133">
         <f t="shared" si="1"/>
         <v>12.818610191887021</v>
       </c>
-      <c r="AD11" s="134">
+      <c r="AD11" s="133">
         <v>250</v>
       </c>
-      <c r="AE11" s="126">
+      <c r="AE11" s="125">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R12" s="118">
+      <c r="R12" s="117">
         <v>80</v>
       </c>
-      <c r="S12" s="131">
+      <c r="S12" s="130">
         <v>13</v>
       </c>
-      <c r="T12" s="132">
+      <c r="T12" s="131">
         <v>16</v>
       </c>
-      <c r="U12" s="132">
+      <c r="U12" s="131">
         <v>19.5</v>
       </c>
-      <c r="V12" s="133">
+      <c r="V12" s="132">
         <v>28</v>
       </c>
-      <c r="AB12" s="135">
+      <c r="AB12" s="134">
         <v>40</v>
       </c>
-      <c r="AC12" s="135">
+      <c r="AC12" s="134">
         <f t="shared" si="1"/>
         <v>15.905414575341014</v>
       </c>
-      <c r="AD12" s="135">
+      <c r="AD12" s="134">
         <v>250</v>
       </c>
-      <c r="AE12" s="129">
+      <c r="AE12" s="128">
         <v>9.5</v>
       </c>
     </row>
     <row r="13" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="AB13" s="135">
+      <c r="AB13" s="134">
         <v>50</v>
       </c>
-      <c r="AC13" s="135">
+      <c r="AC13" s="134">
         <f t="shared" si="1"/>
         <v>18.803015465431965</v>
       </c>
-      <c r="AD13" s="135">
+      <c r="AD13" s="134">
         <v>250</v>
       </c>
-      <c r="AE13" s="129">
+      <c r="AE13" s="128">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="6:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="R14" s="141" t="s">
+      <c r="R14" s="140" t="s">
         <v>394</v>
       </c>
-      <c r="S14" s="119"/>
-      <c r="T14" s="119"/>
-      <c r="U14" s="119"/>
-      <c r="V14" s="119"/>
-      <c r="AB14" s="135">
+      <c r="S14" s="118"/>
+      <c r="T14" s="118"/>
+      <c r="U14" s="118"/>
+      <c r="V14" s="118"/>
+      <c r="AB14" s="134">
         <v>60</v>
       </c>
-      <c r="AC14" s="135">
+      <c r="AC14" s="134">
         <f t="shared" si="1"/>
         <v>21.558246717785043</v>
       </c>
-      <c r="AD14" s="135">
+      <c r="AD14" s="134">
         <v>250</v>
       </c>
-      <c r="AE14" s="129">
+      <c r="AE14" s="128">
         <v>12.5</v>
       </c>
     </row>
     <row r="15" spans="6:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="R15" s="120" t="s">
+      <c r="R15" s="119" t="s">
         <v>355</v>
       </c>
-      <c r="S15" s="120" t="s">
+      <c r="S15" s="119" t="s">
         <v>388</v>
       </c>
-      <c r="T15" s="119"/>
-      <c r="U15" s="119"/>
-      <c r="V15" s="119"/>
-      <c r="AB15" s="135">
+      <c r="T15" s="118"/>
+      <c r="U15" s="118"/>
+      <c r="V15" s="118"/>
+      <c r="AB15" s="134">
         <v>70</v>
       </c>
-      <c r="AC15" s="135">
+      <c r="AC15" s="134">
         <f t="shared" si="1"/>
         <v>24.200454924935883</v>
       </c>
-      <c r="AD15" s="135">
+      <c r="AD15" s="134">
         <v>250</v>
       </c>
-      <c r="AE15" s="129">
+      <c r="AE15" s="128">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="6:31" x14ac:dyDescent="0.25">
-      <c r="R16" s="121" t="s">
+      <c r="R16" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="S16" s="152">
+      <c r="S16" s="151">
         <v>0</v>
       </c>
-      <c r="T16" s="153">
+      <c r="T16" s="152">
         <v>0.25</v>
       </c>
-      <c r="U16" s="153">
+      <c r="U16" s="152">
         <v>0.5</v>
       </c>
-      <c r="V16" s="154">
+      <c r="V16" s="153">
         <v>1</v>
       </c>
-      <c r="AB16" s="136">
+      <c r="AB16" s="135">
         <v>80</v>
       </c>
-      <c r="AC16" s="136">
+      <c r="AC16" s="135">
         <f t="shared" si="1"/>
         <v>26.749612199056873</v>
       </c>
-      <c r="AD16" s="136">
+      <c r="AD16" s="135">
         <v>250</v>
       </c>
-      <c r="AE16" s="132">
+      <c r="AE16" s="131">
         <v>16</v>
       </c>
     </row>
     <row r="17" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R17" s="115">
+      <c r="R17" s="114">
         <v>30</v>
       </c>
-      <c r="S17" s="143">
+      <c r="S17" s="142">
         <f t="shared" ref="S17:V22" si="2">($Y$8+$R17*$Y$9+S$16*$Y$10)/S7</f>
         <v>0.79999999999999993</v>
       </c>
-      <c r="T17" s="144">
+      <c r="T17" s="143">
         <f t="shared" si="2"/>
         <v>0.99062499999999998</v>
       </c>
-      <c r="U17" s="144">
+      <c r="U17" s="143">
         <f t="shared" si="2"/>
         <v>1.0045454545454546</v>
       </c>
-      <c r="V17" s="145">
+      <c r="V17" s="144">
         <f t="shared" si="2"/>
         <v>0.98857142857142866</v>
       </c>
-      <c r="AB17" s="134">
+      <c r="AB17" s="133">
         <v>30</v>
       </c>
-      <c r="AC17" s="134">
+      <c r="AC17" s="133">
         <f t="shared" si="1"/>
         <v>12.818610191887021</v>
       </c>
-      <c r="AD17" s="134">
+      <c r="AD17" s="133">
         <v>500</v>
       </c>
-      <c r="AE17" s="126">
+      <c r="AE17" s="125">
         <v>11</v>
       </c>
     </row>
     <row r="18" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R18" s="117">
+      <c r="R18" s="116">
         <v>40</v>
       </c>
-      <c r="S18" s="146">
+      <c r="S18" s="145">
         <f t="shared" si="2"/>
         <v>0.91428571428571437</v>
       </c>
-      <c r="T18" s="147">
+      <c r="T18" s="146">
         <f>($Y$8+$R18*$Y$9+T$16*$Y$10)/T8</f>
         <v>1.0026315789473685</v>
       </c>
-      <c r="U18" s="147">
+      <c r="U18" s="146">
         <f t="shared" si="2"/>
         <v>1.012</v>
       </c>
-      <c r="V18" s="148">
+      <c r="V18" s="147">
         <f t="shared" si="2"/>
         <v>0.99473684210526303</v>
       </c>
-      <c r="AB18" s="135">
+      <c r="AB18" s="134">
         <v>40</v>
       </c>
-      <c r="AC18" s="135">
+      <c r="AC18" s="134">
         <f t="shared" si="1"/>
         <v>15.905414575341014</v>
       </c>
-      <c r="AD18" s="135">
+      <c r="AD18" s="134">
         <v>500</v>
       </c>
-      <c r="AE18" s="129">
+      <c r="AE18" s="128">
         <v>12.5</v>
       </c>
     </row>
     <row r="19" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R19" s="117">
+      <c r="R19" s="116">
         <v>50</v>
       </c>
-      <c r="S19" s="146">
+      <c r="S19" s="145">
         <f t="shared" si="2"/>
         <v>0.94117647058823528</v>
       </c>
-      <c r="T19" s="147">
+      <c r="T19" s="146">
         <f t="shared" si="2"/>
         <v>1.0113636363636365</v>
       </c>
-      <c r="U19" s="147">
+      <c r="U19" s="146">
         <f t="shared" si="2"/>
         <v>1.0178571428571428</v>
       </c>
-      <c r="V19" s="148">
+      <c r="V19" s="147">
         <f t="shared" si="2"/>
         <v>0.97619047619047616</v>
       </c>
-      <c r="AB19" s="135">
+      <c r="AB19" s="134">
         <v>50</v>
       </c>
-      <c r="AC19" s="135">
+      <c r="AC19" s="134">
         <f t="shared" si="1"/>
         <v>18.803015465431965</v>
       </c>
-      <c r="AD19" s="135">
+      <c r="AD19" s="134">
         <v>500</v>
       </c>
-      <c r="AE19" s="129">
+      <c r="AE19" s="128">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R20" s="117">
+      <c r="R20" s="116">
         <v>60</v>
       </c>
-      <c r="S20" s="146">
+      <c r="S20" s="145">
         <f t="shared" si="2"/>
         <v>0.96</v>
       </c>
-      <c r="T20" s="147">
+      <c r="T20" s="146">
         <f t="shared" si="2"/>
         <v>1.018</v>
       </c>
-      <c r="U20" s="147">
+      <c r="U20" s="146">
         <f t="shared" si="2"/>
         <v>1.0225806451612902</v>
       </c>
-      <c r="V20" s="148">
+      <c r="V20" s="147">
         <f t="shared" si="2"/>
         <v>0.96086956521739142</v>
       </c>
-      <c r="AB20" s="135">
+      <c r="AB20" s="134">
         <v>60</v>
       </c>
-      <c r="AC20" s="135">
+      <c r="AC20" s="134">
         <f t="shared" si="1"/>
         <v>21.558246717785043</v>
       </c>
-      <c r="AD20" s="135">
+      <c r="AD20" s="134">
         <v>500</v>
       </c>
-      <c r="AE20" s="129">
+      <c r="AE20" s="128">
         <v>15.5</v>
       </c>
     </row>
     <row r="21" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R21" s="117">
+      <c r="R21" s="116">
         <v>70</v>
       </c>
-      <c r="S21" s="146">
+      <c r="S21" s="145">
         <f t="shared" si="2"/>
         <v>0.97391304347826091</v>
       </c>
-      <c r="T21" s="147">
+      <c r="T21" s="146">
         <f t="shared" si="2"/>
         <v>1.0232142857142859</v>
       </c>
-      <c r="U21" s="147">
+      <c r="U21" s="146">
         <f t="shared" si="2"/>
         <v>0.99714285714285733</v>
       </c>
-      <c r="V21" s="148">
+      <c r="V21" s="147">
         <f t="shared" si="2"/>
         <v>0.94800000000000006</v>
       </c>
-      <c r="AB21" s="135">
+      <c r="AB21" s="134">
         <v>70</v>
       </c>
-      <c r="AC21" s="135">
+      <c r="AC21" s="134">
         <f t="shared" si="1"/>
         <v>24.200454924935883</v>
       </c>
-      <c r="AD21" s="135">
+      <c r="AD21" s="134">
         <v>500</v>
       </c>
-      <c r="AE21" s="129">
+      <c r="AE21" s="128">
         <v>17.5</v>
       </c>
     </row>
     <row r="22" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R22" s="118">
+      <c r="R22" s="117">
         <v>80</v>
       </c>
-      <c r="S22" s="149">
+      <c r="S22" s="148">
         <f t="shared" si="2"/>
         <v>0.98461538461538467</v>
       </c>
-      <c r="T22" s="150">
+      <c r="T22" s="149">
         <f t="shared" si="2"/>
         <v>0.99531250000000004</v>
       </c>
-      <c r="U22" s="150">
+      <c r="U22" s="149">
         <f t="shared" si="2"/>
         <v>0.97692307692307701</v>
       </c>
-      <c r="V22" s="151">
+      <c r="V22" s="150">
         <f t="shared" si="2"/>
         <v>0.90357142857142858</v>
       </c>
-      <c r="AB22" s="136">
+      <c r="AB22" s="135">
         <v>80</v>
       </c>
-      <c r="AC22" s="136">
+      <c r="AC22" s="135">
         <f t="shared" si="1"/>
         <v>26.749612199056873</v>
       </c>
-      <c r="AD22" s="136">
+      <c r="AD22" s="135">
         <v>500</v>
       </c>
-      <c r="AE22" s="132">
+      <c r="AE22" s="131">
         <v>19.5</v>
       </c>
     </row>
     <row r="23" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="AB23" s="134">
+      <c r="AB23" s="133">
         <v>30</v>
       </c>
-      <c r="AC23" s="134">
+      <c r="AC23" s="133">
         <f t="shared" si="1"/>
         <v>12.818610191887021</v>
       </c>
-      <c r="AD23" s="134">
+      <c r="AD23" s="133">
         <v>1000</v>
       </c>
-      <c r="AE23" s="126">
+      <c r="AE23" s="125">
         <v>17.5</v>
       </c>
     </row>
     <row r="24" spans="18:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="R24" s="141" t="s">
+      <c r="R24" s="140" t="s">
         <v>393</v>
       </c>
-      <c r="S24" s="119"/>
-      <c r="T24" s="119"/>
-      <c r="U24" s="119"/>
-      <c r="V24" s="119"/>
-      <c r="AB24" s="135">
+      <c r="S24" s="118"/>
+      <c r="T24" s="118"/>
+      <c r="U24" s="118"/>
+      <c r="V24" s="118"/>
+      <c r="AB24" s="134">
         <v>40</v>
       </c>
-      <c r="AC24" s="135">
+      <c r="AC24" s="134">
         <f t="shared" si="1"/>
         <v>15.905414575341014</v>
       </c>
-      <c r="AD24" s="135">
+      <c r="AD24" s="134">
         <v>1000</v>
       </c>
-      <c r="AE24" s="129">
+      <c r="AE24" s="128">
         <v>19</v>
       </c>
     </row>
     <row r="25" spans="18:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="R25" s="120" t="s">
+      <c r="R25" s="119" t="s">
         <v>355</v>
       </c>
-      <c r="S25" s="120" t="s">
+      <c r="S25" s="119" t="s">
         <v>388</v>
       </c>
-      <c r="T25" s="119"/>
-      <c r="U25" s="119"/>
-      <c r="V25" s="119"/>
-      <c r="AB25" s="135">
+      <c r="T25" s="118"/>
+      <c r="U25" s="118"/>
+      <c r="V25" s="118"/>
+      <c r="AB25" s="134">
         <v>50</v>
       </c>
-      <c r="AC25" s="135">
+      <c r="AC25" s="134">
         <f t="shared" si="1"/>
         <v>18.803015465431965</v>
       </c>
-      <c r="AD25" s="135">
+      <c r="AD25" s="134">
         <v>1000</v>
       </c>
-      <c r="AE25" s="129">
+      <c r="AE25" s="128">
         <v>21</v>
       </c>
     </row>
     <row r="26" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R26" s="121" t="s">
+      <c r="R26" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="S26" s="152">
+      <c r="S26" s="151">
         <v>0</v>
       </c>
-      <c r="T26" s="153">
+      <c r="T26" s="152">
         <v>0.25</v>
       </c>
-      <c r="U26" s="153">
+      <c r="U26" s="152">
         <v>0.5</v>
       </c>
-      <c r="V26" s="154">
+      <c r="V26" s="153">
         <v>1</v>
       </c>
-      <c r="AB26" s="135">
+      <c r="AB26" s="134">
         <v>60</v>
       </c>
-      <c r="AC26" s="135">
+      <c r="AC26" s="134">
         <f t="shared" si="1"/>
         <v>21.558246717785043</v>
       </c>
-      <c r="AD26" s="135">
+      <c r="AD26" s="134">
         <v>1000</v>
       </c>
-      <c r="AE26" s="129">
+      <c r="AE26" s="128">
         <v>23</v>
       </c>
     </row>
     <row r="27" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R27" s="115">
+      <c r="R27" s="114">
         <v>30</v>
       </c>
-      <c r="S27" s="143">
+      <c r="S27" s="142">
         <f>(0.475*$R27^0.75 + S$26*$X$27)/S7</f>
         <v>1.0148066401910558</v>
       </c>
-      <c r="T27" s="144">
+      <c r="T27" s="143">
         <f t="shared" ref="T27:V27" si="3">(0.475*$R27^0.75 + T$26*$X$27)/T7</f>
         <v>1.1361049801432919</v>
       </c>
-      <c r="U27" s="144">
+      <c r="U27" s="143">
         <f t="shared" si="3"/>
         <v>1.0989854401042123</v>
       </c>
-      <c r="V27" s="145">
+      <c r="V27" s="144">
         <f t="shared" si="3"/>
         <v>1.0336479909226477</v>
       </c>
       <c r="X27">
         <v>12</v>
       </c>
-      <c r="AB27" s="135">
+      <c r="AB27" s="134">
         <v>70</v>
       </c>
-      <c r="AC27" s="135">
+      <c r="AC27" s="134">
         <f t="shared" si="1"/>
         <v>24.200454924935883</v>
       </c>
-      <c r="AD27" s="135">
+      <c r="AD27" s="134">
         <v>1000</v>
       </c>
-      <c r="AE27" s="129">
+      <c r="AE27" s="128">
         <v>25</v>
       </c>
     </row>
     <row r="28" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R28" s="117">
+      <c r="R28" s="116">
         <v>40</v>
       </c>
-      <c r="S28" s="146">
+      <c r="S28" s="145">
         <f t="shared" ref="S28:V28" si="4">(0.475*$R28^0.75 + S$26*$X$27)/S8</f>
         <v>1.0792959890409974</v>
       </c>
-      <c r="T28" s="147">
+      <c r="T28" s="146">
         <f t="shared" si="4"/>
         <v>1.1110602024512612</v>
       </c>
-      <c r="U28" s="147">
+      <c r="U28" s="146">
         <f t="shared" si="4"/>
         <v>1.0844057538629586</v>
       </c>
-      <c r="V28" s="148">
+      <c r="V28" s="147">
         <f t="shared" si="4"/>
         <v>1.0292143117519463</v>
       </c>
       <c r="X28">
         <v>0.2</v>
       </c>
-      <c r="AB28" s="136">
+      <c r="AB28" s="135">
         <v>80</v>
       </c>
-      <c r="AC28" s="136">
+      <c r="AC28" s="135">
         <f t="shared" si="1"/>
         <v>26.749612199056873</v>
       </c>
-      <c r="AD28" s="136">
+      <c r="AD28" s="135">
         <v>1000</v>
       </c>
-      <c r="AE28" s="132">
+      <c r="AE28" s="131">
         <v>28</v>
       </c>
     </row>
     <row r="29" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R29" s="117">
+      <c r="R29" s="116">
         <v>50</v>
       </c>
-      <c r="S29" s="146">
+      <c r="S29" s="145">
         <f t="shared" ref="S29:V29" si="5">(0.475*$R29^0.75 + S$26*$X$27)/S9</f>
         <v>1.0507567465976686</v>
       </c>
-      <c r="T29" s="147">
+      <c r="T29" s="146">
         <f t="shared" si="5"/>
         <v>1.0846756678254712</v>
       </c>
-      <c r="U29" s="147">
+      <c r="U29" s="146">
         <f t="shared" si="5"/>
         <v>1.0665308818628703</v>
       </c>
-      <c r="V29" s="148">
+      <c r="V29" s="147">
         <f t="shared" si="5"/>
         <v>0.99673487362286584</v>
       </c>
     </row>
     <row r="30" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R30" s="117">
+      <c r="R30" s="116">
         <v>60</v>
       </c>
-      <c r="S30" s="146">
+      <c r="S30" s="145">
         <f t="shared" ref="S30:V30" si="6">(0.475*$R30^0.75 + S$26*$X$27)/S10</f>
         <v>1.0240167190947895</v>
       </c>
-      <c r="T30" s="147">
+      <c r="T30" s="146">
         <f t="shared" si="6"/>
         <v>1.0592133752758317</v>
       </c>
-      <c r="U30" s="147">
+      <c r="U30" s="146">
         <f t="shared" si="6"/>
         <v>1.0477527219966383</v>
       </c>
-      <c r="V30" s="148">
+      <c r="V30" s="147">
         <f t="shared" si="6"/>
         <v>0.966963790910778</v>
       </c>
     </row>
     <row r="31" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R31" s="117">
+      <c r="R31" s="116">
         <v>70</v>
       </c>
-      <c r="S31" s="146">
+      <c r="S31" s="145">
         <f t="shared" ref="S31:V31" si="7">(0.475*$R31^0.75 + S$26*$X$27)/S11</f>
         <v>0.99958400776909073</v>
       </c>
-      <c r="T31" s="147">
+      <c r="T31" s="146">
         <f t="shared" si="7"/>
         <v>1.0353725778103244</v>
       </c>
-      <c r="U31" s="147">
+      <c r="U31" s="146">
         <f t="shared" si="7"/>
         <v>0.99972663367683112</v>
       </c>
-      <c r="V31" s="148">
+      <c r="V31" s="147">
         <f t="shared" si="7"/>
         <v>0.9398086435737818</v>
       </c>
     </row>
     <row r="32" spans="18:31" x14ac:dyDescent="0.25">
-      <c r="R32" s="118">
+      <c r="R32" s="117">
         <v>80</v>
       </c>
-      <c r="S32" s="149">
+      <c r="S32" s="148">
         <f t="shared" ref="S32:V32" si="8">(0.475*$R32^0.75 + S$26*$X$27)/S12</f>
         <v>0.9773896765040011</v>
       </c>
-      <c r="T32" s="150">
+      <c r="T32" s="149">
         <f t="shared" si="8"/>
         <v>0.98162911215950088</v>
       </c>
-      <c r="U32" s="150">
+      <c r="U32" s="149">
         <f t="shared" si="8"/>
         <v>0.95928542536164174</v>
       </c>
-      <c r="V32" s="151">
+      <c r="V32" s="150">
         <f t="shared" si="8"/>
         <v>0.88235949266257196</v>
       </c>

</xml_diff>

<commit_message>
Added fallback parameter values to avoid warnings and cleaned notebook
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -56,13 +56,13 @@
   </definedNames>
   <calcPr calcId="162913" iterate="1"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId12"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="435">
   <si>
     <t>value</t>
   </si>
@@ -2236,7 +2236,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2490,6 +2490,7 @@
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -14002,7 +14003,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L3:O43" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField axis="axisRow" showAll="0">
@@ -16280,7 +16281,7 @@
       <c r="H30" t="s">
         <v>407</v>
       </c>
-      <c r="I30">
+      <c r="I30" s="93">
         <v>0</v>
       </c>
       <c r="J30" t="s">
@@ -16297,7 +16298,7 @@
       <c r="H31" t="s">
         <v>407</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="93">
         <v>0</v>
       </c>
       <c r="J31" t="s">
@@ -16440,6 +16441,15 @@
       <c r="B41" t="s">
         <v>1</v>
       </c>
+      <c r="H41" t="s">
+        <v>407</v>
+      </c>
+      <c r="I41" s="93">
+        <v>0</v>
+      </c>
+      <c r="J41" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
@@ -16447,6 +16457,15 @@
       </c>
       <c r="B42" t="s">
         <v>5</v>
+      </c>
+      <c r="H42" t="s">
+        <v>407</v>
+      </c>
+      <c r="I42" s="93">
+        <v>0</v>
+      </c>
+      <c r="J42" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -16911,6 +16930,18 @@
       </c>
       <c r="L62" t="s">
         <v>333</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H63" s="160" t="s">
+        <v>301</v>
+      </c>
+      <c r="I63" s="160">
+        <v>0</v>
+      </c>
+      <c r="J63" s="160"/>
+      <c r="K63" s="161" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fixed GeoDistributor C2 speed and how domestic/regional feeds are handled + Start working on pig feed rations
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -54,7 +54,7 @@
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
   </definedNames>
-  <calcPr calcId="162913" iterate="1"/>
+  <calcPr calcId="162913" iterate="1" calcCompleted="0"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId12"/>
   </pivotCaches>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="435">
   <si>
     <t>value</t>
   </si>
@@ -18590,37 +18590,32 @@
       <c r="L153" s="95"/>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A154" s="97" t="s">
+      <c r="H154" s="160" t="s">
+        <v>327</v>
+      </c>
+      <c r="I154" s="160">
+        <v>0</v>
+      </c>
+      <c r="J154" s="160"/>
+      <c r="K154" s="160" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A155" s="97" t="s">
         <v>304</v>
       </c>
-      <c r="B154" s="97"/>
-      <c r="C154" s="97"/>
-      <c r="D154" s="98"/>
-      <c r="E154" s="98"/>
-      <c r="F154" s="98"/>
-      <c r="G154" s="98"/>
-      <c r="H154" s="98"/>
-      <c r="I154" s="99"/>
-      <c r="J154" s="98"/>
-      <c r="K154" s="98"/>
-      <c r="L154" s="98"/>
-    </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
-        <v>2</v>
-      </c>
-      <c r="D155" t="s">
-        <v>18</v>
-      </c>
-      <c r="E155" t="s">
-        <v>329</v>
-      </c>
-      <c r="H155" t="s">
-        <v>327</v>
-      </c>
-      <c r="I155">
-        <v>40</v>
-      </c>
+      <c r="B155" s="97"/>
+      <c r="C155" s="97"/>
+      <c r="D155" s="98"/>
+      <c r="E155" s="98"/>
+      <c r="F155" s="98"/>
+      <c r="G155" s="98"/>
+      <c r="H155" s="98"/>
+      <c r="I155" s="99"/>
+      <c r="J155" s="98"/>
+      <c r="K155" s="98"/>
+      <c r="L155" s="98"/>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
@@ -18630,13 +18625,13 @@
         <v>18</v>
       </c>
       <c r="E156" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
       <c r="H156" t="s">
         <v>327</v>
       </c>
       <c r="I156">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
@@ -18647,13 +18642,13 @@
         <v>18</v>
       </c>
       <c r="E157" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="H157" t="s">
         <v>327</v>
       </c>
       <c r="I157">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
@@ -18664,27 +18659,30 @@
         <v>18</v>
       </c>
       <c r="E158" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="H158" t="s">
         <v>327</v>
       </c>
       <c r="I158">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>2</v>
       </c>
+      <c r="D159" t="s">
+        <v>18</v>
+      </c>
       <c r="E159" t="s">
-        <v>329</v>
+        <v>397</v>
       </c>
       <c r="H159" t="s">
         <v>327</v>
       </c>
       <c r="I159">
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
@@ -18692,13 +18690,13 @@
         <v>2</v>
       </c>
       <c r="E160" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
       <c r="H160" t="s">
         <v>327</v>
       </c>
       <c r="I160">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
@@ -18706,7 +18704,7 @@
         <v>2</v>
       </c>
       <c r="E161" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="H161" t="s">
         <v>327</v>
@@ -18720,30 +18718,27 @@
         <v>2</v>
       </c>
       <c r="E162" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="H162" t="s">
         <v>327</v>
       </c>
       <c r="I162">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>2</v>
       </c>
-      <c r="D163" t="s">
-        <v>35</v>
-      </c>
       <c r="E163" t="s">
-        <v>329</v>
+        <v>397</v>
       </c>
       <c r="H163" t="s">
         <v>327</v>
       </c>
       <c r="I163">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
@@ -18754,13 +18749,13 @@
         <v>35</v>
       </c>
       <c r="E164" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
       <c r="H164" t="s">
         <v>327</v>
       </c>
       <c r="I164">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
@@ -18771,13 +18766,13 @@
         <v>35</v>
       </c>
       <c r="E165" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="H165" t="s">
         <v>327</v>
       </c>
       <c r="I165">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
@@ -18788,63 +18783,60 @@
         <v>35</v>
       </c>
       <c r="E166" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="H166" t="s">
         <v>327</v>
       </c>
       <c r="I166">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>2</v>
+      </c>
+      <c r="D167" t="s">
+        <v>35</v>
+      </c>
+      <c r="E167" t="s">
+        <v>397</v>
+      </c>
+      <c r="H167" t="s">
+        <v>327</v>
+      </c>
+      <c r="I167">
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A168" s="100" t="s">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A169" s="100" t="s">
         <v>305</v>
       </c>
-      <c r="B168" s="100"/>
-      <c r="C168" s="100"/>
-      <c r="D168" s="101"/>
-      <c r="E168" s="101"/>
-      <c r="F168" s="101"/>
-      <c r="G168" s="101"/>
-      <c r="H168" s="101"/>
-      <c r="I168" s="101"/>
-      <c r="J168" s="101"/>
-      <c r="K168" s="101"/>
-      <c r="L168" s="101"/>
-    </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
-        <v>39</v>
-      </c>
-      <c r="E169" t="s">
-        <v>329</v>
-      </c>
-      <c r="H169" t="s">
-        <v>327</v>
-      </c>
-      <c r="I169">
-        <v>60</v>
-      </c>
-      <c r="J169" t="s">
-        <v>328</v>
-      </c>
+      <c r="B169" s="100"/>
+      <c r="C169" s="100"/>
+      <c r="D169" s="101"/>
+      <c r="E169" s="101"/>
+      <c r="F169" s="101"/>
+      <c r="G169" s="101"/>
+      <c r="H169" s="101"/>
+      <c r="I169" s="101"/>
+      <c r="J169" s="101"/>
+      <c r="K169" s="101"/>
+      <c r="L169" s="101"/>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>39</v>
       </c>
       <c r="E170" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
       <c r="H170" t="s">
         <v>327</v>
       </c>
       <c r="I170">
-        <v>30</v>
-      </c>
-      <c r="J170" t="s">
-        <v>328</v>
+        <v>60</v>
       </c>
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.25">
@@ -18852,36 +18844,27 @@
         <v>39</v>
       </c>
       <c r="E171" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="H171" t="s">
         <v>327</v>
       </c>
       <c r="I171">
-        <v>10</v>
-      </c>
-      <c r="J171" t="s">
-        <v>328</v>
+        <v>30</v>
       </c>
     </row>
     <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>39</v>
       </c>
-      <c r="D172" t="s">
-        <v>35</v>
-      </c>
       <c r="E172" t="s">
-        <v>329</v>
+        <v>399</v>
       </c>
       <c r="H172" t="s">
         <v>327</v>
       </c>
       <c r="I172">
-        <v>50</v>
-      </c>
-      <c r="J172" t="s">
-        <v>328</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173" spans="1:12" x14ac:dyDescent="0.25">
@@ -18892,16 +18875,13 @@
         <v>35</v>
       </c>
       <c r="E173" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
       <c r="H173" t="s">
         <v>327</v>
       </c>
       <c r="I173">
-        <v>0</v>
-      </c>
-      <c r="J173" t="s">
-        <v>328</v>
+        <v>50</v>
       </c>
     </row>
     <row r="174" spans="1:12" x14ac:dyDescent="0.25">
@@ -18912,30 +18892,30 @@
         <v>35</v>
       </c>
       <c r="E174" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="H174" t="s">
         <v>327</v>
       </c>
       <c r="I174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>39</v>
+      </c>
+      <c r="D175" t="s">
+        <v>35</v>
+      </c>
+      <c r="E175" t="s">
+        <v>399</v>
+      </c>
+      <c r="H175" t="s">
+        <v>327</v>
+      </c>
+      <c r="I175">
         <v>50</v>
-      </c>
-      <c r="J174" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H176" s="160" t="s">
-        <v>327</v>
-      </c>
-      <c r="I176" s="160">
-        <v>0</v>
-      </c>
-      <c r="J176" s="160" t="s">
-        <v>328</v>
-      </c>
-      <c r="K176" s="160" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
@@ -18990,9 +18970,10 @@
       <c r="H180" t="s">
         <v>433</v>
       </c>
-      <c r="J180" s="93">
+      <c r="I180" s="93">
         <v>5</v>
       </c>
+      <c r="J180" s="93"/>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
@@ -19004,9 +18985,10 @@
       <c r="H181" t="s">
         <v>433</v>
       </c>
-      <c r="J181" s="93">
+      <c r="I181" s="93">
         <v>5</v>
       </c>
+      <c r="J181" s="93"/>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
@@ -19018,9 +19000,10 @@
       <c r="H182" t="s">
         <v>433</v>
       </c>
-      <c r="J182" s="93">
+      <c r="I182" s="93">
         <v>0</v>
       </c>
+      <c r="J182" s="93"/>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
@@ -19032,9 +19015,10 @@
       <c r="H183" t="s">
         <v>433</v>
       </c>
-      <c r="J183" s="93">
+      <c r="I183" s="93">
         <v>100</v>
       </c>
+      <c r="J183" s="93"/>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
@@ -19046,9 +19030,10 @@
       <c r="H184" t="s">
         <v>433</v>
       </c>
-      <c r="J184" s="93">
+      <c r="I184" s="93">
         <v>100</v>
       </c>
+      <c r="J184" s="93"/>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
@@ -19060,9 +19045,10 @@
       <c r="H185" t="s">
         <v>433</v>
       </c>
-      <c r="J185" s="93">
+      <c r="I185" s="93">
         <v>0</v>
       </c>
+      <c r="J185" s="93"/>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" s="100" t="s">
@@ -19090,9 +19076,10 @@
       <c r="H188" t="s">
         <v>433</v>
       </c>
-      <c r="J188" s="93">
+      <c r="I188" s="93">
         <v>100</v>
       </c>
+      <c r="J188" s="93"/>
     </row>
     <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
@@ -19104,9 +19091,10 @@
       <c r="H189" t="s">
         <v>433</v>
       </c>
-      <c r="J189" s="93">
+      <c r="I189" s="93">
         <v>100</v>
       </c>
+      <c r="J189" s="93"/>
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
@@ -19118,9 +19106,10 @@
       <c r="H190" t="s">
         <v>433</v>
       </c>
-      <c r="J190" s="93">
+      <c r="I190" s="93">
         <v>0</v>
       </c>
+      <c r="J190" s="93"/>
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
@@ -19132,9 +19121,10 @@
       <c r="H191" t="s">
         <v>433</v>
       </c>
-      <c r="J191" s="93">
+      <c r="I191" s="93">
         <v>100</v>
       </c>
+      <c r="J191" s="93"/>
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
@@ -19146,9 +19136,10 @@
       <c r="H192" t="s">
         <v>433</v>
       </c>
-      <c r="J192" s="93">
+      <c r="I192" s="93">
         <v>100</v>
       </c>
+      <c r="J192" s="93"/>
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
@@ -19160,9 +19151,10 @@
       <c r="H193" t="s">
         <v>433</v>
       </c>
-      <c r="J193" s="93">
+      <c r="I193" s="93">
         <v>100</v>
       </c>
+      <c r="J193" s="93"/>
     </row>
     <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" s="159" t="s">

</xml_diff>

<commit_message>
Updated dairy cow feed rations and implementd 'maize based' sub_system + various fixes to make the sub_system implementation work
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -54,7 +54,7 @@
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
   </definedNames>
-  <calcPr calcId="162913" iterate="1" calcCompleted="0"/>
+  <calcPr calcId="162913" iterate="1"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId12"/>
   </pivotCaches>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2543" uniqueCount="442">
   <si>
     <t>value</t>
   </si>
@@ -1267,13 +1267,7 @@
     <t>Total incl. for calves</t>
   </si>
   <si>
-    <t>rapeseed meal/cake</t>
-  </si>
-  <si>
     <t>f_sub_system</t>
-  </si>
-  <si>
-    <t>wheat</t>
   </si>
   <si>
     <t>Avg</t>
@@ -1379,6 +1373,33 @@
   </si>
   <si>
     <t>This parameter specifies the maximum share of grazing demand that can be met from grazing in semi-natural grasslands</t>
+  </si>
+  <si>
+    <t>straw</t>
+  </si>
+  <si>
+    <t>barley</t>
+  </si>
+  <si>
+    <t>rapeseed meal</t>
+  </si>
+  <si>
+    <t>wheat distillers grain, dry</t>
+  </si>
+  <si>
+    <t>maize based</t>
+  </si>
+  <si>
+    <t>maize silage</t>
+  </si>
+  <si>
+    <t>sugar beet pulp</t>
+  </si>
+  <si>
+    <t>wheat bran</t>
+  </si>
+  <si>
+    <t>Mikaela Lindberg (SLU) pers. com. 2023-04-21</t>
   </si>
 </sst>
 </file>
@@ -15723,7 +15744,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:L201"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -15748,7 +15769,7 @@
         <v>296</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>53</v>
@@ -16279,13 +16300,13 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="I30" s="93">
         <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -16296,13 +16317,13 @@
         <v>5</v>
       </c>
       <c r="H31" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="I31" s="93">
         <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -16442,13 +16463,13 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="I41" s="93">
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -16459,13 +16480,13 @@
         <v>5</v>
       </c>
       <c r="H42" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="I42" s="93">
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -16941,7 +16962,7 @@
       </c>
       <c r="J63" s="160"/>
       <c r="K63" s="161" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -17582,7 +17603,7 @@
         <v>2</v>
       </c>
       <c r="D99" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H99" t="s">
         <v>36</v>
@@ -17614,7 +17635,7 @@
         <v>9</v>
       </c>
       <c r="K100" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
@@ -17637,7 +17658,7 @@
         <v>9</v>
       </c>
       <c r="K101" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
@@ -17660,7 +17681,7 @@
         <v>9</v>
       </c>
       <c r="K102" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
@@ -17683,7 +17704,7 @@
         <v>9</v>
       </c>
       <c r="K103" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
@@ -17706,7 +17727,7 @@
         <v>9</v>
       </c>
       <c r="K104" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
@@ -17729,7 +17750,7 @@
         <v>9</v>
       </c>
       <c r="K105" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
@@ -17752,7 +17773,7 @@
         <v>9</v>
       </c>
       <c r="K106" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
@@ -17775,7 +17796,7 @@
         <v>9</v>
       </c>
       <c r="K107" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
@@ -17969,7 +17990,7 @@
         <v>39</v>
       </c>
       <c r="D119" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H119" t="s">
         <v>36</v>
@@ -18001,7 +18022,7 @@
         <v>9</v>
       </c>
       <c r="K120" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
@@ -18024,7 +18045,7 @@
         <v>9</v>
       </c>
       <c r="K121" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
@@ -18047,7 +18068,7 @@
         <v>9</v>
       </c>
       <c r="K122" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -18070,7 +18091,7 @@
         <v>9</v>
       </c>
       <c r="K123" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
@@ -18093,7 +18114,7 @@
         <v>9</v>
       </c>
       <c r="K124" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
@@ -18116,7 +18137,7 @@
         <v>9</v>
       </c>
       <c r="K125" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -18139,7 +18160,7 @@
         <v>9</v>
       </c>
       <c r="K126" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
@@ -18162,7 +18183,7 @@
         <v>9</v>
       </c>
       <c r="K127" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.25">
@@ -18307,7 +18328,7 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="94" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B137" s="94"/>
       <c r="C137" s="94"/>
@@ -18326,30 +18347,30 @@
         <v>18</v>
       </c>
       <c r="H138" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="I138">
         <v>0.50700000000000001</v>
       </c>
       <c r="J138" t="s">
+        <v>411</v>
+      </c>
+      <c r="L138" t="s">
         <v>413</v>
-      </c>
-      <c r="L138" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H139" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="I139">
         <v>0.47499999999999998</v>
       </c>
       <c r="J139" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="L139" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
@@ -18357,16 +18378,16 @@
         <v>18</v>
       </c>
       <c r="H140" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="I140" s="13">
         <v>5</v>
       </c>
       <c r="J140" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="L140" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.25">
@@ -18377,20 +18398,20 @@
         <v>18</v>
       </c>
       <c r="H141" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="I141" s="13">
         <f>(0.013+0.021+0.038) * 30.4</f>
         <v>2.1888000000000001</v>
       </c>
       <c r="J141" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="K141" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="L141" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.25">
@@ -18401,31 +18422,31 @@
         <v>18</v>
       </c>
       <c r="H142" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="I142" s="13">
         <f>(8 * 7 * 3.6)/100</f>
         <v>2.016</v>
       </c>
       <c r="J142" t="s">
+        <v>416</v>
+      </c>
+      <c r="K142" t="s">
         <v>418</v>
       </c>
-      <c r="K142" t="s">
-        <v>420</v>
-      </c>
       <c r="L142" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H143" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I143" s="1">
         <v>1</v>
       </c>
       <c r="J143" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.25">
@@ -18436,16 +18457,16 @@
         <v>18</v>
       </c>
       <c r="H144" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I144" s="1">
         <v>1.1100000000000001</v>
       </c>
       <c r="J144" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L144" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
@@ -18456,19 +18477,19 @@
         <v>35</v>
       </c>
       <c r="H145" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I145" s="1">
         <v>0.9</v>
       </c>
       <c r="J145" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="K145" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="L145" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.25">
@@ -18476,16 +18497,16 @@
         <v>33</v>
       </c>
       <c r="H146" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I146" s="1">
         <v>1.05</v>
       </c>
       <c r="J146" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L146" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
@@ -18496,27 +18517,27 @@
         <v>34</v>
       </c>
       <c r="H147" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I147" s="1">
         <v>1.05</v>
       </c>
       <c r="J147" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L147" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H148" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I148" s="13">
         <v>0</v>
       </c>
       <c r="J148" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.25">
@@ -18527,16 +18548,16 @@
         <v>18</v>
       </c>
       <c r="H149" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I149" s="13">
         <v>-13.6</v>
       </c>
       <c r="J149" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L149" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.25">
@@ -18573,7 +18594,7 @@
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="94" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B153" s="94"/>
       <c r="C153" s="94"/>
@@ -18598,7 +18619,7 @@
       </c>
       <c r="J154" s="160"/>
       <c r="K154" s="160" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
@@ -18631,7 +18652,10 @@
         <v>327</v>
       </c>
       <c r="I156">
-        <v>40</v>
+        <v>48</v>
+      </c>
+      <c r="L156" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
@@ -18642,13 +18666,16 @@
         <v>18</v>
       </c>
       <c r="E157" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="H157" t="s">
         <v>327</v>
       </c>
       <c r="I157">
         <v>10</v>
+      </c>
+      <c r="L157" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
@@ -18659,13 +18686,16 @@
         <v>18</v>
       </c>
       <c r="E158" t="s">
-        <v>399</v>
+        <v>433</v>
       </c>
       <c r="H158" t="s">
         <v>327</v>
       </c>
       <c r="I158">
-        <v>35</v>
+        <v>3</v>
+      </c>
+      <c r="L158" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
@@ -18676,639 +18706,889 @@
         <v>18</v>
       </c>
       <c r="E159" t="s">
-        <v>397</v>
+        <v>434</v>
       </c>
       <c r="H159" t="s">
         <v>327</v>
       </c>
       <c r="I159">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="L159" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>2</v>
       </c>
+      <c r="D160" t="s">
+        <v>18</v>
+      </c>
       <c r="E160" t="s">
-        <v>329</v>
+        <v>435</v>
       </c>
       <c r="H160" t="s">
         <v>327</v>
       </c>
       <c r="I160">
-        <v>50</v>
+        <v>6</v>
+      </c>
+      <c r="L160" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>2</v>
       </c>
+      <c r="D161" t="s">
+        <v>18</v>
+      </c>
       <c r="E161" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="H161" t="s">
         <v>327</v>
       </c>
       <c r="I161">
-        <v>25</v>
+        <v>8</v>
+      </c>
+      <c r="L161" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>2</v>
       </c>
+      <c r="C162" t="s">
+        <v>437</v>
+      </c>
+      <c r="D162" t="s">
+        <v>18</v>
+      </c>
       <c r="E162" t="s">
-        <v>399</v>
+        <v>329</v>
       </c>
       <c r="H162" t="s">
         <v>327</v>
       </c>
       <c r="I162">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="L162" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>2</v>
       </c>
+      <c r="C163" t="s">
+        <v>437</v>
+      </c>
+      <c r="D163" t="s">
+        <v>18</v>
+      </c>
       <c r="E163" t="s">
-        <v>397</v>
+        <v>438</v>
       </c>
       <c r="H163" t="s">
         <v>327</v>
       </c>
       <c r="I163">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="L163" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>2</v>
       </c>
+      <c r="C164" t="s">
+        <v>437</v>
+      </c>
       <c r="D164" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E164" t="s">
-        <v>329</v>
+        <v>427</v>
       </c>
       <c r="H164" t="s">
         <v>327</v>
       </c>
       <c r="I164">
-        <v>50</v>
+        <v>10</v>
+      </c>
+      <c r="L164" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>2</v>
       </c>
+      <c r="C165" t="s">
+        <v>437</v>
+      </c>
       <c r="D165" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E165" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="H165" t="s">
         <v>327</v>
       </c>
       <c r="I165">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="L165" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>2</v>
       </c>
+      <c r="C166" t="s">
+        <v>437</v>
+      </c>
       <c r="D166" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E166" t="s">
-        <v>399</v>
+        <v>434</v>
       </c>
       <c r="H166" t="s">
         <v>327</v>
       </c>
       <c r="I166">
-        <v>50</v>
+        <v>17</v>
+      </c>
+      <c r="L166" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>2</v>
       </c>
+      <c r="C167" t="s">
+        <v>437</v>
+      </c>
       <c r="D167" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E167" t="s">
-        <v>397</v>
+        <v>435</v>
       </c>
       <c r="H167" t="s">
         <v>327</v>
       </c>
       <c r="I167">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="L167" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>2</v>
+      </c>
+      <c r="C168" t="s">
+        <v>437</v>
+      </c>
+      <c r="D168" t="s">
+        <v>18</v>
+      </c>
+      <c r="E168" t="s">
+        <v>436</v>
+      </c>
+      <c r="H168" t="s">
+        <v>327</v>
+      </c>
+      <c r="I168">
+        <v>9</v>
+      </c>
+      <c r="L168" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="169" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A169" s="100" t="s">
-        <v>305</v>
-      </c>
-      <c r="B169" s="100"/>
-      <c r="C169" s="100"/>
-      <c r="D169" s="101"/>
-      <c r="E169" s="101"/>
-      <c r="F169" s="101"/>
-      <c r="G169" s="101"/>
-      <c r="H169" s="101"/>
-      <c r="I169" s="101"/>
-      <c r="J169" s="101"/>
-      <c r="K169" s="101"/>
-      <c r="L169" s="101"/>
+      <c r="A169" t="s">
+        <v>2</v>
+      </c>
+      <c r="C169" t="s">
+        <v>437</v>
+      </c>
+      <c r="D169" t="s">
+        <v>18</v>
+      </c>
+      <c r="E169" t="s">
+        <v>439</v>
+      </c>
+      <c r="H169" t="s">
+        <v>327</v>
+      </c>
+      <c r="I169">
+        <v>5</v>
+      </c>
+      <c r="L169" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>39</v>
+        <v>2</v>
+      </c>
+      <c r="C170" t="s">
+        <v>437</v>
+      </c>
+      <c r="D170" t="s">
+        <v>18</v>
       </c>
       <c r="E170" t="s">
-        <v>329</v>
+        <v>440</v>
       </c>
       <c r="H170" t="s">
         <v>327</v>
       </c>
       <c r="I170">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>39</v>
-      </c>
-      <c r="E171" t="s">
-        <v>429</v>
-      </c>
-      <c r="H171" t="s">
-        <v>327</v>
-      </c>
-      <c r="I171">
-        <v>30</v>
+        <v>1</v>
+      </c>
+      <c r="L170" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="E172" t="s">
-        <v>399</v>
+        <v>329</v>
       </c>
       <c r="H172" t="s">
         <v>327</v>
       </c>
       <c r="I172">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>39</v>
-      </c>
-      <c r="D173" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E173" t="s">
-        <v>329</v>
+        <v>427</v>
       </c>
       <c r="H173" t="s">
         <v>327</v>
       </c>
       <c r="I173">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>39</v>
-      </c>
-      <c r="D174" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E174" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="H174" t="s">
         <v>327</v>
       </c>
       <c r="I174">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>39</v>
-      </c>
-      <c r="D175" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E175" t="s">
-        <v>399</v>
+        <v>435</v>
       </c>
       <c r="H175" t="s">
         <v>327</v>
       </c>
       <c r="I175">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>2</v>
+      </c>
+      <c r="D176" t="s">
+        <v>35</v>
+      </c>
+      <c r="E176" t="s">
+        <v>329</v>
+      </c>
+      <c r="H176" t="s">
+        <v>327</v>
+      </c>
+      <c r="I176">
         <v>50</v>
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H177" s="93"/>
-      <c r="I177" s="93"/>
-      <c r="J177" s="93"/>
-      <c r="K177" s="93"/>
+      <c r="A177" t="s">
+        <v>2</v>
+      </c>
+      <c r="D177" t="s">
+        <v>35</v>
+      </c>
+      <c r="E177" t="s">
+        <v>427</v>
+      </c>
+      <c r="H177" t="s">
+        <v>327</v>
+      </c>
+      <c r="I177">
+        <v>0</v>
+      </c>
     </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A178" s="94" t="s">
-        <v>432</v>
-      </c>
-      <c r="B178" s="94"/>
-      <c r="C178" s="94"/>
-      <c r="D178" s="95"/>
-      <c r="E178" s="95"/>
-      <c r="F178" s="95"/>
-      <c r="G178" s="95"/>
-      <c r="H178" s="95"/>
-      <c r="I178" s="95"/>
-      <c r="J178" s="95" t="s">
-        <v>9</v>
-      </c>
-      <c r="K178" s="95" t="s">
+      <c r="A178" t="s">
+        <v>2</v>
+      </c>
+      <c r="D178" t="s">
+        <v>35</v>
+      </c>
+      <c r="E178" t="s">
         <v>434</v>
       </c>
-      <c r="L178" s="95"/>
+      <c r="H178" t="s">
+        <v>327</v>
+      </c>
+      <c r="I178">
+        <v>50</v>
+      </c>
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A179" s="97" t="s">
-        <v>304</v>
-      </c>
-      <c r="B179" s="97"/>
-      <c r="C179" s="97"/>
-      <c r="D179" s="98"/>
-      <c r="E179" s="98"/>
-      <c r="F179" s="98"/>
-      <c r="G179" s="98"/>
-      <c r="H179" s="98"/>
-      <c r="I179" s="99"/>
-      <c r="J179" s="98"/>
-      <c r="K179" s="98"/>
-      <c r="L179" s="98"/>
-    </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
+      <c r="A179" t="s">
         <v>2</v>
       </c>
-      <c r="D180" t="s">
-        <v>18</v>
-      </c>
-      <c r="H180" t="s">
-        <v>433</v>
-      </c>
-      <c r="I180" s="93">
-        <v>5</v>
-      </c>
-      <c r="J180" s="93"/>
+      <c r="D179" t="s">
+        <v>35</v>
+      </c>
+      <c r="E179" t="s">
+        <v>435</v>
+      </c>
+      <c r="H179" t="s">
+        <v>327</v>
+      </c>
+      <c r="I179">
+        <v>0</v>
+      </c>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>2</v>
-      </c>
-      <c r="D181" t="s">
-        <v>20</v>
-      </c>
-      <c r="H181" t="s">
-        <v>433</v>
-      </c>
-      <c r="I181" s="93">
-        <v>5</v>
-      </c>
-      <c r="J181" s="93"/>
+      <c r="A181" s="100" t="s">
+        <v>305</v>
+      </c>
+      <c r="B181" s="100"/>
+      <c r="C181" s="100"/>
+      <c r="D181" s="101"/>
+      <c r="E181" s="101"/>
+      <c r="F181" s="101"/>
+      <c r="G181" s="101"/>
+      <c r="H181" s="101"/>
+      <c r="I181" s="101"/>
+      <c r="J181" s="101"/>
+      <c r="K181" s="101"/>
+      <c r="L181" s="101"/>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>2</v>
-      </c>
-      <c r="D182" t="s">
-        <v>35</v>
+        <v>39</v>
+      </c>
+      <c r="E182" t="s">
+        <v>329</v>
       </c>
       <c r="H182" t="s">
-        <v>433</v>
-      </c>
-      <c r="I182" s="93">
-        <v>0</v>
-      </c>
-      <c r="J182" s="93"/>
+        <v>327</v>
+      </c>
+      <c r="I182">
+        <v>60</v>
+      </c>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>2</v>
-      </c>
-      <c r="D183" t="s">
-        <v>33</v>
+        <v>39</v>
+      </c>
+      <c r="E183" t="s">
+        <v>427</v>
       </c>
       <c r="H183" t="s">
-        <v>433</v>
-      </c>
-      <c r="I183" s="93">
-        <v>100</v>
-      </c>
-      <c r="J183" s="93"/>
+        <v>327</v>
+      </c>
+      <c r="I183">
+        <v>30</v>
+      </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>2</v>
-      </c>
-      <c r="D184" t="s">
-        <v>34</v>
+        <v>39</v>
+      </c>
+      <c r="E184" t="s">
+        <v>434</v>
       </c>
       <c r="H184" t="s">
-        <v>433</v>
-      </c>
-      <c r="I184" s="93">
-        <v>100</v>
-      </c>
-      <c r="J184" s="93"/>
+        <v>327</v>
+      </c>
+      <c r="I184">
+        <v>10</v>
+      </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="D185" t="s">
-        <v>431</v>
+        <v>35</v>
+      </c>
+      <c r="E185" t="s">
+        <v>329</v>
       </c>
       <c r="H185" t="s">
-        <v>433</v>
-      </c>
-      <c r="I185" s="93">
+        <v>327</v>
+      </c>
+      <c r="I185">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>39</v>
+      </c>
+      <c r="D186" t="s">
+        <v>35</v>
+      </c>
+      <c r="E186" t="s">
+        <v>427</v>
+      </c>
+      <c r="H186" t="s">
+        <v>327</v>
+      </c>
+      <c r="I186">
         <v>0</v>
       </c>
-      <c r="J185" s="93"/>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A187" s="100" t="s">
-        <v>305</v>
-      </c>
-      <c r="B187" s="100"/>
-      <c r="C187" s="100"/>
-      <c r="D187" s="101"/>
-      <c r="E187" s="101"/>
-      <c r="F187" s="101"/>
-      <c r="G187" s="101"/>
-      <c r="H187" s="101"/>
-      <c r="I187" s="101"/>
-      <c r="J187" s="101"/>
-      <c r="K187" s="101"/>
-      <c r="L187" s="101"/>
-    </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
+      <c r="A187" t="s">
         <v>39</v>
       </c>
-      <c r="D188" t="s">
-        <v>18</v>
-      </c>
-      <c r="H188" t="s">
-        <v>433</v>
-      </c>
-      <c r="I188" s="93">
-        <v>100</v>
-      </c>
-      <c r="J188" s="93"/>
+      <c r="D187" t="s">
+        <v>35</v>
+      </c>
+      <c r="E187" t="s">
+        <v>434</v>
+      </c>
+      <c r="H187" t="s">
+        <v>327</v>
+      </c>
+      <c r="I187">
+        <v>50</v>
+      </c>
     </row>
     <row r="189" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
-        <v>39</v>
-      </c>
-      <c r="D189" t="s">
-        <v>20</v>
-      </c>
-      <c r="H189" t="s">
-        <v>433</v>
-      </c>
-      <c r="I189" s="93">
-        <v>100</v>
-      </c>
+      <c r="H189" s="93"/>
+      <c r="I189" s="93"/>
       <c r="J189" s="93"/>
+      <c r="K189" s="93"/>
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A190" t="s">
-        <v>39</v>
-      </c>
-      <c r="D190" t="s">
-        <v>35</v>
-      </c>
-      <c r="H190" t="s">
-        <v>433</v>
-      </c>
-      <c r="I190" s="93">
-        <v>0</v>
-      </c>
-      <c r="J190" s="93"/>
+      <c r="A190" s="94" t="s">
+        <v>430</v>
+      </c>
+      <c r="B190" s="94"/>
+      <c r="C190" s="94"/>
+      <c r="D190" s="95"/>
+      <c r="E190" s="95"/>
+      <c r="F190" s="95"/>
+      <c r="G190" s="95"/>
+      <c r="H190" s="95"/>
+      <c r="I190" s="95"/>
+      <c r="J190" s="95" t="s">
+        <v>9</v>
+      </c>
+      <c r="K190" s="95" t="s">
+        <v>432</v>
+      </c>
+      <c r="L190" s="95"/>
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A191" t="s">
-        <v>39</v>
-      </c>
-      <c r="D191" t="s">
-        <v>33</v>
-      </c>
-      <c r="H191" t="s">
-        <v>433</v>
-      </c>
-      <c r="I191" s="93">
-        <v>100</v>
-      </c>
-      <c r="J191" s="93"/>
+      <c r="A191" s="97" t="s">
+        <v>304</v>
+      </c>
+      <c r="B191" s="97"/>
+      <c r="C191" s="97"/>
+      <c r="D191" s="98"/>
+      <c r="E191" s="98"/>
+      <c r="F191" s="98"/>
+      <c r="G191" s="98"/>
+      <c r="H191" s="98"/>
+      <c r="I191" s="99"/>
+      <c r="J191" s="98"/>
+      <c r="K191" s="98"/>
+      <c r="L191" s="98"/>
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="D192" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="H192" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="I192" s="93">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="J192" s="93"/>
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
+        <v>2</v>
+      </c>
+      <c r="D193" t="s">
+        <v>20</v>
+      </c>
+      <c r="H193" t="s">
+        <v>431</v>
+      </c>
+      <c r="I193" s="93">
+        <v>5</v>
+      </c>
+      <c r="J193" s="93"/>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>2</v>
+      </c>
+      <c r="D194" t="s">
+        <v>35</v>
+      </c>
+      <c r="H194" t="s">
+        <v>431</v>
+      </c>
+      <c r="I194" s="93">
+        <v>0</v>
+      </c>
+      <c r="J194" s="93"/>
+    </row>
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>2</v>
+      </c>
+      <c r="D195" t="s">
+        <v>33</v>
+      </c>
+      <c r="H195" t="s">
+        <v>431</v>
+      </c>
+      <c r="I195" s="93">
+        <v>100</v>
+      </c>
+      <c r="J195" s="93"/>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>2</v>
+      </c>
+      <c r="D196" t="s">
+        <v>34</v>
+      </c>
+      <c r="H196" t="s">
+        <v>431</v>
+      </c>
+      <c r="I196" s="93">
+        <v>100</v>
+      </c>
+      <c r="J196" s="93"/>
+    </row>
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>2</v>
+      </c>
+      <c r="D197" t="s">
+        <v>429</v>
+      </c>
+      <c r="H197" t="s">
+        <v>431</v>
+      </c>
+      <c r="I197" s="93">
+        <v>0</v>
+      </c>
+      <c r="J197" s="93"/>
+    </row>
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A199" s="100" t="s">
+        <v>305</v>
+      </c>
+      <c r="B199" s="100"/>
+      <c r="C199" s="100"/>
+      <c r="D199" s="101"/>
+      <c r="E199" s="101"/>
+      <c r="F199" s="101"/>
+      <c r="G199" s="101"/>
+      <c r="H199" s="101"/>
+      <c r="I199" s="101"/>
+      <c r="J199" s="101"/>
+      <c r="K199" s="101"/>
+      <c r="L199" s="101"/>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
         <v>39</v>
       </c>
-      <c r="D193" t="s">
+      <c r="D200" t="s">
+        <v>18</v>
+      </c>
+      <c r="H200" t="s">
         <v>431</v>
       </c>
-      <c r="H193" t="s">
-        <v>433</v>
-      </c>
-      <c r="I193" s="93">
+      <c r="I200" s="93">
         <v>100</v>
       </c>
-      <c r="J193" s="93"/>
-    </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A195" s="159" t="s">
+      <c r="J200" s="93"/>
+    </row>
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>39</v>
+      </c>
+      <c r="D201" t="s">
+        <v>20</v>
+      </c>
+      <c r="H201" t="s">
+        <v>431</v>
+      </c>
+      <c r="I201" s="93">
+        <v>100</v>
+      </c>
+      <c r="J201" s="93"/>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>39</v>
+      </c>
+      <c r="D202" t="s">
+        <v>35</v>
+      </c>
+      <c r="H202" t="s">
+        <v>431</v>
+      </c>
+      <c r="I202" s="93">
+        <v>0</v>
+      </c>
+      <c r="J202" s="93"/>
+    </row>
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>39</v>
+      </c>
+      <c r="D203" t="s">
+        <v>33</v>
+      </c>
+      <c r="H203" t="s">
+        <v>431</v>
+      </c>
+      <c r="I203" s="93">
+        <v>100</v>
+      </c>
+      <c r="J203" s="93"/>
+    </row>
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>39</v>
+      </c>
+      <c r="D204" t="s">
+        <v>34</v>
+      </c>
+      <c r="H204" t="s">
+        <v>431</v>
+      </c>
+      <c r="I204" s="93">
+        <v>100</v>
+      </c>
+      <c r="J204" s="93"/>
+    </row>
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>39</v>
+      </c>
+      <c r="D205" t="s">
+        <v>429</v>
+      </c>
+      <c r="H205" t="s">
+        <v>431</v>
+      </c>
+      <c r="I205" s="93">
+        <v>100</v>
+      </c>
+      <c r="J205" s="93"/>
+    </row>
+    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A207" s="159" t="s">
         <v>306</v>
       </c>
-      <c r="B195" s="159"/>
-      <c r="C195" s="159"/>
-      <c r="D195" s="95"/>
-      <c r="E195" s="95"/>
-      <c r="F195" s="95"/>
-      <c r="G195" s="95"/>
-      <c r="H195" s="95"/>
-      <c r="I195" s="95"/>
-      <c r="J195" s="95"/>
-      <c r="K195" s="95"/>
-      <c r="L195" s="95"/>
-    </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A196" s="93" t="s">
+      <c r="B207" s="159"/>
+      <c r="C207" s="159"/>
+      <c r="D207" s="95"/>
+      <c r="E207" s="95"/>
+      <c r="F207" s="95"/>
+      <c r="G207" s="95"/>
+      <c r="H207" s="95"/>
+      <c r="I207" s="95"/>
+      <c r="J207" s="95"/>
+      <c r="K207" s="95"/>
+      <c r="L207" s="95"/>
+    </row>
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A208" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D196" s="93" t="s">
+      <c r="D208" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="E196" s="93"/>
-      <c r="F196" s="93"/>
-      <c r="G196" s="93"/>
-      <c r="H196" s="93" t="s">
+      <c r="E208" s="93"/>
+      <c r="F208" s="93"/>
+      <c r="G208" s="93"/>
+      <c r="H208" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I196" s="93">
+      <c r="I208" s="93">
         <v>7.1</v>
       </c>
-      <c r="J196" s="93" t="s">
+      <c r="J208" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K196" s="93"/>
-      <c r="L196" s="93" t="s">
+      <c r="K208" s="93"/>
+      <c r="L208" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A197" s="93" t="s">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A209" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="D197" s="93" t="s">
+      <c r="D209" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="E197" s="93"/>
-      <c r="F197" s="93"/>
-      <c r="G197" s="93"/>
-      <c r="H197" s="93" t="s">
+      <c r="E209" s="93"/>
+      <c r="F209" s="93"/>
+      <c r="G209" s="93"/>
+      <c r="H209" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I197" s="93">
+      <c r="I209" s="93">
         <v>5.0999999999999996</v>
       </c>
-      <c r="J197" s="93" t="s">
+      <c r="J209" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K197" s="93"/>
-      <c r="L197" s="93" t="s">
+      <c r="K209" s="93"/>
+      <c r="L209" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A198" s="93"/>
-      <c r="D198" s="93" t="s">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A210" s="93"/>
+      <c r="D210" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="E198" s="93"/>
-      <c r="F198" s="93"/>
-      <c r="G198" s="93"/>
-      <c r="H198" s="93" t="s">
+      <c r="E210" s="93"/>
+      <c r="F210" s="93"/>
+      <c r="G210" s="93"/>
+      <c r="H210" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I198" s="93">
+      <c r="I210" s="93">
         <v>5.7</v>
       </c>
-      <c r="J198" s="93" t="s">
+      <c r="J210" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K198" s="93"/>
-      <c r="L198" s="93" t="s">
+      <c r="K210" s="93"/>
+      <c r="L210" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A199" s="93"/>
-      <c r="D199" s="93" t="s">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A211" s="93"/>
+      <c r="D211" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="E199" s="93"/>
-      <c r="F199" s="93"/>
-      <c r="G199" s="93"/>
-      <c r="H199" s="93" t="s">
+      <c r="E211" s="93"/>
+      <c r="F211" s="93"/>
+      <c r="G211" s="93"/>
+      <c r="H211" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I199" s="93">
+      <c r="I211" s="93">
         <v>7.7</v>
       </c>
-      <c r="J199" s="93" t="s">
+      <c r="J211" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K199" s="93"/>
-      <c r="L199" s="93" t="s">
+      <c r="K211" s="93"/>
+      <c r="L211" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A200" s="93"/>
-      <c r="D200" s="93" t="s">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A212" s="93"/>
+      <c r="D212" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="E200" s="93"/>
-      <c r="F200" s="93"/>
-      <c r="G200" s="93"/>
-      <c r="H200" s="93" t="s">
+      <c r="E212" s="93"/>
+      <c r="F212" s="93"/>
+      <c r="G212" s="93"/>
+      <c r="H212" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I200" s="93">
+      <c r="I212" s="93">
         <v>9.1</v>
       </c>
-      <c r="J200" s="93" t="s">
+      <c r="J212" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K200" s="93" t="s">
+      <c r="K212" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="L200" s="93" t="s">
+      <c r="L212" s="93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A201" s="93"/>
-      <c r="D201" s="93" t="s">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A213" s="93"/>
+      <c r="D213" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E201" s="93"/>
-      <c r="F201" s="93"/>
-      <c r="G201" s="93"/>
-      <c r="H201" s="93" t="s">
+      <c r="E213" s="93"/>
+      <c r="F213" s="93"/>
+      <c r="G213" s="93"/>
+      <c r="H213" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="I201" s="93">
+      <c r="I213" s="93">
         <v>9.1</v>
       </c>
-      <c r="J201" s="93" t="s">
+      <c r="J213" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="K201" s="93" t="s">
+      <c r="K213" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="L201" s="93" t="s">
+      <c r="L213" s="93" t="s">
         <v>42</v>
       </c>
     </row>
@@ -25167,7 +25447,7 @@
     </row>
     <row r="96" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="98" spans="2:11" x14ac:dyDescent="0.25">
@@ -25175,10 +25455,10 @@
         <v>317</v>
       </c>
       <c r="F98" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="I98" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="99" spans="2:11" x14ac:dyDescent="0.25">
@@ -25186,28 +25466,28 @@
         <v>18</v>
       </c>
       <c r="D99" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E99" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F99" t="s">
         <v>18</v>
       </c>
       <c r="G99" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="H99" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="I99" t="s">
         <v>18</v>
       </c>
       <c r="J99" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K99" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.25">
@@ -25397,7 +25677,7 @@
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B105" s="155" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C105" s="2">
         <f>AVERAGE(C100:C104)</f>
@@ -25438,7 +25718,7 @@
     </row>
     <row r="106" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D106" s="155" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E106" s="156">
         <f>1/E105</f>

</xml_diff>

<commit_message>
changes to baseline scenario
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="13" r:id="rId1"/>
@@ -57,7 +57,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId13"/>
+    <pivotCache cacheId="0" r:id="rId13"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -14549,7 +14549,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L3:O43" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField axis="axisRow" showAll="0">
@@ -25458,7 +25458,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
@@ -25512,30 +25512,38 @@
         <v>1</v>
       </c>
       <c r="E2" s="1">
-        <f>D2*1.06</f>
-        <v>1.06</v>
+        <f>D2*1.01^5</f>
+        <v>1.0510100500999999</v>
       </c>
       <c r="F2" s="1">
-        <f t="shared" ref="F2:J2" si="0">E2*1.06</f>
-        <v>1.1236000000000002</v>
+        <f>E2*1.0081^5</f>
+        <v>1.0942711329791557</v>
       </c>
       <c r="G2" s="1">
-        <f t="shared" si="0"/>
-        <v>1.1910160000000003</v>
+        <f>F2*1.0061^5</f>
+        <v>1.1280560721959558</v>
       </c>
       <c r="H2" s="1">
-        <f t="shared" si="0"/>
-        <v>1.2624769600000003</v>
+        <f>G2*1.004^5</f>
+        <v>1.1507984060123795</v>
       </c>
       <c r="I2" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3382255776000005</v>
+        <f>H2*1.002^5</f>
+        <v>1.1623525141647169</v>
       </c>
       <c r="J2" s="1">
-        <f t="shared" si="0"/>
-        <v>1.4185191122560006</v>
+        <f>I2*1.001^5</f>
+        <v>1.1681759118900195</v>
       </c>
       <c r="K2" s="2"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Created function to automatically instantiate AnimalHerd objects
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3696" uniqueCount="541">
   <si>
     <t>value</t>
   </si>
@@ -20602,7 +20602,9 @@
       <c r="A179" s="159" t="s">
         <v>2</v>
       </c>
-      <c r="B179" s="159"/>
+      <c r="B179" s="159" t="s">
+        <v>1</v>
+      </c>
       <c r="C179" s="159" t="s">
         <v>432</v>
       </c>
@@ -20624,6 +20626,9 @@
       <c r="A180" t="s">
         <v>2</v>
       </c>
+      <c r="B180" t="s">
+        <v>1</v>
+      </c>
       <c r="C180" t="s">
         <v>432</v>
       </c>
@@ -20647,6 +20652,9 @@
       <c r="A181" t="s">
         <v>2</v>
       </c>
+      <c r="B181" t="s">
+        <v>1</v>
+      </c>
       <c r="C181" t="s">
         <v>432</v>
       </c>
@@ -20670,6 +20678,9 @@
       <c r="A182" t="s">
         <v>2</v>
       </c>
+      <c r="B182" t="s">
+        <v>1</v>
+      </c>
       <c r="C182" t="s">
         <v>432</v>
       </c>
@@ -20693,6 +20704,9 @@
       <c r="A183" t="s">
         <v>2</v>
       </c>
+      <c r="B183" t="s">
+        <v>1</v>
+      </c>
       <c r="C183" t="s">
         <v>432</v>
       </c>
@@ -20716,6 +20730,9 @@
       <c r="A184" t="s">
         <v>2</v>
       </c>
+      <c r="B184" t="s">
+        <v>1</v>
+      </c>
       <c r="C184" t="s">
         <v>432</v>
       </c>
@@ -20739,6 +20756,9 @@
       <c r="A185" t="s">
         <v>2</v>
       </c>
+      <c r="B185" t="s">
+        <v>1</v>
+      </c>
       <c r="C185" t="s">
         <v>432</v>
       </c>
@@ -20762,6 +20782,9 @@
       <c r="A186" t="s">
         <v>2</v>
       </c>
+      <c r="B186" t="s">
+        <v>1</v>
+      </c>
       <c r="C186" t="s">
         <v>432</v>
       </c>
@@ -20785,6 +20808,9 @@
       <c r="A187" t="s">
         <v>2</v>
       </c>
+      <c r="B187" t="s">
+        <v>1</v>
+      </c>
       <c r="C187" t="s">
         <v>432</v>
       </c>
@@ -20808,6 +20834,9 @@
       <c r="A188" t="s">
         <v>2</v>
       </c>
+      <c r="B188" t="s">
+        <v>1</v>
+      </c>
       <c r="C188" t="s">
         <v>432</v>
       </c>
@@ -20831,6 +20860,9 @@
       <c r="A189" t="s">
         <v>2</v>
       </c>
+      <c r="B189" t="s">
+        <v>1</v>
+      </c>
       <c r="C189" t="s">
         <v>432</v>
       </c>
@@ -20854,6 +20886,9 @@
       <c r="A190" t="s">
         <v>2</v>
       </c>
+      <c r="B190" t="s">
+        <v>1</v>
+      </c>
       <c r="C190" t="s">
         <v>432</v>
       </c>
@@ -20877,6 +20912,9 @@
       <c r="A191" t="s">
         <v>2</v>
       </c>
+      <c r="B191" t="s">
+        <v>1</v>
+      </c>
       <c r="C191" t="s">
         <v>432</v>
       </c>
@@ -20900,6 +20938,9 @@
       <c r="A192" t="s">
         <v>2</v>
       </c>
+      <c r="B192" t="s">
+        <v>1</v>
+      </c>
       <c r="C192" t="s">
         <v>432</v>
       </c>
@@ -20923,6 +20964,9 @@
       <c r="A193" t="s">
         <v>2</v>
       </c>
+      <c r="B193" t="s">
+        <v>1</v>
+      </c>
       <c r="C193" t="s">
         <v>432</v>
       </c>
@@ -20946,6 +20990,9 @@
       <c r="A194" t="s">
         <v>2</v>
       </c>
+      <c r="B194" t="s">
+        <v>1</v>
+      </c>
       <c r="C194" t="s">
         <v>432</v>
       </c>
@@ -20969,6 +21016,9 @@
       <c r="A195" t="s">
         <v>2</v>
       </c>
+      <c r="B195" t="s">
+        <v>1</v>
+      </c>
       <c r="C195" t="s">
         <v>432</v>
       </c>
@@ -20992,6 +21042,9 @@
       <c r="A196" t="s">
         <v>2</v>
       </c>
+      <c r="B196" t="s">
+        <v>1</v>
+      </c>
       <c r="C196" t="s">
         <v>432</v>
       </c>
@@ -21015,6 +21068,9 @@
       <c r="A197" t="s">
         <v>2</v>
       </c>
+      <c r="B197" t="s">
+        <v>1</v>
+      </c>
       <c r="C197" t="s">
         <v>432</v>
       </c>
@@ -21038,6 +21094,9 @@
       <c r="A198" t="s">
         <v>2</v>
       </c>
+      <c r="B198" t="s">
+        <v>1</v>
+      </c>
       <c r="C198" t="s">
         <v>432</v>
       </c>
@@ -21061,6 +21120,9 @@
       <c r="A199" t="s">
         <v>2</v>
       </c>
+      <c r="B199" t="s">
+        <v>1</v>
+      </c>
       <c r="C199" t="s">
         <v>432</v>
       </c>
@@ -21084,6 +21146,9 @@
       <c r="A200" t="s">
         <v>2</v>
       </c>
+      <c r="B200" t="s">
+        <v>1</v>
+      </c>
       <c r="C200" t="s">
         <v>432</v>
       </c>
@@ -21107,6 +21172,9 @@
       <c r="A201" t="s">
         <v>2</v>
       </c>
+      <c r="B201" t="s">
+        <v>1</v>
+      </c>
       <c r="C201" t="s">
         <v>432</v>
       </c>
@@ -21128,6 +21196,9 @@
       <c r="A202" t="s">
         <v>2</v>
       </c>
+      <c r="B202" t="s">
+        <v>1</v>
+      </c>
       <c r="C202" t="s">
         <v>432</v>
       </c>
@@ -21149,6 +21220,9 @@
       <c r="A203" t="s">
         <v>2</v>
       </c>
+      <c r="B203" t="s">
+        <v>1</v>
+      </c>
       <c r="C203" t="s">
         <v>432</v>
       </c>
@@ -21170,6 +21244,9 @@
       <c r="A204" t="s">
         <v>2</v>
       </c>
+      <c r="B204" t="s">
+        <v>1</v>
+      </c>
       <c r="C204" t="s">
         <v>432</v>
       </c>
@@ -21191,6 +21268,9 @@
       <c r="A205" t="s">
         <v>2</v>
       </c>
+      <c r="B205" t="s">
+        <v>1</v>
+      </c>
       <c r="C205" t="s">
         <v>432</v>
       </c>
@@ -21212,6 +21292,9 @@
       <c r="A206" t="s">
         <v>2</v>
       </c>
+      <c r="B206" t="s">
+        <v>1</v>
+      </c>
       <c r="C206" t="s">
         <v>432</v>
       </c>
@@ -21232,6 +21315,9 @@
     <row r="207" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>2</v>
+      </c>
+      <c r="B207" t="s">
+        <v>1</v>
       </c>
       <c r="C207" t="s">
         <v>432</v>
@@ -22342,7 +22428,9 @@
       <c r="A271" s="159" t="s">
         <v>2</v>
       </c>
-      <c r="B271" s="159"/>
+      <c r="B271" s="159" t="s">
+        <v>1</v>
+      </c>
       <c r="C271" s="159" t="s">
         <v>432</v>
       </c>
@@ -22364,6 +22452,9 @@
       <c r="A272" t="s">
         <v>2</v>
       </c>
+      <c r="B272" t="s">
+        <v>1</v>
+      </c>
       <c r="C272" t="s">
         <v>432</v>
       </c>
@@ -22387,6 +22478,9 @@
       <c r="A273" t="s">
         <v>2</v>
       </c>
+      <c r="B273" t="s">
+        <v>1</v>
+      </c>
       <c r="C273" t="s">
         <v>432</v>
       </c>
@@ -22410,6 +22504,9 @@
       <c r="A274" t="s">
         <v>2</v>
       </c>
+      <c r="B274" t="s">
+        <v>1</v>
+      </c>
       <c r="C274" t="s">
         <v>432</v>
       </c>
@@ -22433,6 +22530,9 @@
       <c r="A275" t="s">
         <v>2</v>
       </c>
+      <c r="B275" t="s">
+        <v>1</v>
+      </c>
       <c r="C275" t="s">
         <v>432</v>
       </c>
@@ -22456,6 +22556,9 @@
       <c r="A276" t="s">
         <v>2</v>
       </c>
+      <c r="B276" t="s">
+        <v>1</v>
+      </c>
       <c r="C276" t="s">
         <v>432</v>
       </c>
@@ -22479,6 +22582,9 @@
       <c r="A277" t="s">
         <v>2</v>
       </c>
+      <c r="B277" t="s">
+        <v>1</v>
+      </c>
       <c r="C277" t="s">
         <v>432</v>
       </c>
@@ -22502,6 +22608,9 @@
       <c r="A278" t="s">
         <v>2</v>
       </c>
+      <c r="B278" t="s">
+        <v>1</v>
+      </c>
       <c r="C278" t="s">
         <v>432</v>
       </c>
@@ -22525,6 +22634,9 @@
       <c r="A279" t="s">
         <v>2</v>
       </c>
+      <c r="B279" t="s">
+        <v>1</v>
+      </c>
       <c r="C279" t="s">
         <v>432</v>
       </c>
@@ -22548,6 +22660,9 @@
       <c r="A280" t="s">
         <v>2</v>
       </c>
+      <c r="B280" t="s">
+        <v>1</v>
+      </c>
       <c r="C280" t="s">
         <v>432</v>
       </c>
@@ -22571,6 +22686,9 @@
       <c r="A281" t="s">
         <v>2</v>
       </c>
+      <c r="B281" t="s">
+        <v>1</v>
+      </c>
       <c r="C281" t="s">
         <v>432</v>
       </c>
@@ -22594,6 +22712,9 @@
       <c r="A282" t="s">
         <v>2</v>
       </c>
+      <c r="B282" t="s">
+        <v>1</v>
+      </c>
       <c r="C282" t="s">
         <v>432</v>
       </c>
@@ -22617,6 +22738,9 @@
       <c r="A283" t="s">
         <v>2</v>
       </c>
+      <c r="B283" t="s">
+        <v>1</v>
+      </c>
       <c r="C283" t="s">
         <v>432</v>
       </c>
@@ -22640,6 +22764,9 @@
       <c r="A284" t="s">
         <v>2</v>
       </c>
+      <c r="B284" t="s">
+        <v>1</v>
+      </c>
       <c r="C284" t="s">
         <v>432</v>
       </c>
@@ -22663,6 +22790,9 @@
       <c r="A285" t="s">
         <v>2</v>
       </c>
+      <c r="B285" t="s">
+        <v>1</v>
+      </c>
       <c r="C285" t="s">
         <v>432</v>
       </c>
@@ -22686,6 +22816,9 @@
       <c r="A286" t="s">
         <v>2</v>
       </c>
+      <c r="B286" t="s">
+        <v>1</v>
+      </c>
       <c r="C286" t="s">
         <v>432</v>
       </c>
@@ -22709,6 +22842,9 @@
       <c r="A287" t="s">
         <v>2</v>
       </c>
+      <c r="B287" t="s">
+        <v>1</v>
+      </c>
       <c r="C287" t="s">
         <v>432</v>
       </c>
@@ -22732,6 +22868,9 @@
       <c r="A288" t="s">
         <v>2</v>
       </c>
+      <c r="B288" t="s">
+        <v>1</v>
+      </c>
       <c r="C288" t="s">
         <v>432</v>
       </c>
@@ -22755,6 +22894,9 @@
       <c r="A289" t="s">
         <v>2</v>
       </c>
+      <c r="B289" t="s">
+        <v>1</v>
+      </c>
       <c r="C289" t="s">
         <v>432</v>
       </c>
@@ -22778,6 +22920,9 @@
       <c r="A290" t="s">
         <v>2</v>
       </c>
+      <c r="B290" t="s">
+        <v>1</v>
+      </c>
       <c r="C290" t="s">
         <v>432</v>
       </c>
@@ -22801,6 +22946,9 @@
       <c r="A291" t="s">
         <v>2</v>
       </c>
+      <c r="B291" t="s">
+        <v>1</v>
+      </c>
       <c r="C291" t="s">
         <v>432</v>
       </c>
@@ -22824,6 +22972,9 @@
       <c r="A292" t="s">
         <v>2</v>
       </c>
+      <c r="B292" t="s">
+        <v>1</v>
+      </c>
       <c r="C292" t="s">
         <v>432</v>
       </c>
@@ -22847,6 +22998,9 @@
       <c r="A293" t="s">
         <v>2</v>
       </c>
+      <c r="B293" t="s">
+        <v>1</v>
+      </c>
       <c r="C293" t="s">
         <v>432</v>
       </c>
@@ -22868,6 +23022,9 @@
       <c r="A294" t="s">
         <v>2</v>
       </c>
+      <c r="B294" t="s">
+        <v>1</v>
+      </c>
       <c r="C294" t="s">
         <v>432</v>
       </c>
@@ -22889,6 +23046,9 @@
       <c r="A295" t="s">
         <v>2</v>
       </c>
+      <c r="B295" t="s">
+        <v>1</v>
+      </c>
       <c r="C295" t="s">
         <v>432</v>
       </c>
@@ -22910,6 +23070,9 @@
       <c r="A296" t="s">
         <v>2</v>
       </c>
+      <c r="B296" t="s">
+        <v>1</v>
+      </c>
       <c r="C296" t="s">
         <v>432</v>
       </c>
@@ -22931,6 +23094,9 @@
       <c r="A297" t="s">
         <v>2</v>
       </c>
+      <c r="B297" t="s">
+        <v>1</v>
+      </c>
       <c r="C297" t="s">
         <v>432</v>
       </c>
@@ -22952,6 +23118,9 @@
       <c r="A298" t="s">
         <v>2</v>
       </c>
+      <c r="B298" t="s">
+        <v>1</v>
+      </c>
       <c r="C298" t="s">
         <v>432</v>
       </c>
@@ -22972,6 +23141,9 @@
     <row r="299" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>2</v>
+      </c>
+      <c r="B299" t="s">
+        <v>1</v>
       </c>
       <c r="C299" t="s">
         <v>432</v>
@@ -24674,7 +24846,9 @@
       <c r="A395" s="159" t="s">
         <v>38</v>
       </c>
-      <c r="B395" s="159"/>
+      <c r="B395" s="159" t="s">
+        <v>1</v>
+      </c>
       <c r="C395" s="159" t="s">
         <v>432</v>
       </c>
@@ -24696,6 +24870,9 @@
       <c r="A396" t="s">
         <v>38</v>
       </c>
+      <c r="B396" t="s">
+        <v>1</v>
+      </c>
       <c r="C396" t="s">
         <v>432</v>
       </c>
@@ -24719,6 +24896,9 @@
       <c r="A397" t="s">
         <v>38</v>
       </c>
+      <c r="B397" t="s">
+        <v>1</v>
+      </c>
       <c r="C397" t="s">
         <v>432</v>
       </c>
@@ -24742,6 +24922,9 @@
       <c r="A398" t="s">
         <v>38</v>
       </c>
+      <c r="B398" t="s">
+        <v>1</v>
+      </c>
       <c r="C398" t="s">
         <v>432</v>
       </c>
@@ -24765,6 +24948,9 @@
       <c r="A399" t="s">
         <v>38</v>
       </c>
+      <c r="B399" t="s">
+        <v>1</v>
+      </c>
       <c r="C399" t="s">
         <v>432</v>
       </c>
@@ -24788,6 +24974,9 @@
       <c r="A400" t="s">
         <v>38</v>
       </c>
+      <c r="B400" t="s">
+        <v>1</v>
+      </c>
       <c r="C400" t="s">
         <v>432</v>
       </c>
@@ -24811,6 +25000,9 @@
       <c r="A401" t="s">
         <v>38</v>
       </c>
+      <c r="B401" t="s">
+        <v>1</v>
+      </c>
       <c r="C401" t="s">
         <v>432</v>
       </c>
@@ -24834,6 +25026,9 @@
       <c r="A402" t="s">
         <v>38</v>
       </c>
+      <c r="B402" t="s">
+        <v>1</v>
+      </c>
       <c r="C402" t="s">
         <v>432</v>
       </c>
@@ -24857,6 +25052,9 @@
       <c r="A403" t="s">
         <v>38</v>
       </c>
+      <c r="B403" t="s">
+        <v>1</v>
+      </c>
       <c r="C403" t="s">
         <v>432</v>
       </c>
@@ -24880,6 +25078,9 @@
       <c r="A404" t="s">
         <v>38</v>
       </c>
+      <c r="B404" t="s">
+        <v>1</v>
+      </c>
       <c r="C404" t="s">
         <v>432</v>
       </c>
@@ -24903,6 +25104,9 @@
       <c r="A405" t="s">
         <v>38</v>
       </c>
+      <c r="B405" t="s">
+        <v>1</v>
+      </c>
       <c r="C405" t="s">
         <v>432</v>
       </c>
@@ -24926,6 +25130,9 @@
       <c r="A406" t="s">
         <v>38</v>
       </c>
+      <c r="B406" t="s">
+        <v>1</v>
+      </c>
       <c r="C406" t="s">
         <v>432</v>
       </c>
@@ -24949,6 +25156,9 @@
       <c r="A407" t="s">
         <v>38</v>
       </c>
+      <c r="B407" t="s">
+        <v>1</v>
+      </c>
       <c r="C407" t="s">
         <v>432</v>
       </c>
@@ -24972,6 +25182,9 @@
       <c r="A408" t="s">
         <v>38</v>
       </c>
+      <c r="B408" t="s">
+        <v>1</v>
+      </c>
       <c r="C408" t="s">
         <v>432</v>
       </c>
@@ -24995,6 +25208,9 @@
       <c r="A409" t="s">
         <v>38</v>
       </c>
+      <c r="B409" t="s">
+        <v>1</v>
+      </c>
       <c r="C409" t="s">
         <v>432</v>
       </c>
@@ -25018,6 +25234,9 @@
       <c r="A410" t="s">
         <v>38</v>
       </c>
+      <c r="B410" t="s">
+        <v>1</v>
+      </c>
       <c r="C410" t="s">
         <v>432</v>
       </c>
@@ -25041,6 +25260,9 @@
       <c r="A411" t="s">
         <v>38</v>
       </c>
+      <c r="B411" t="s">
+        <v>1</v>
+      </c>
       <c r="C411" t="s">
         <v>432</v>
       </c>
@@ -25064,6 +25286,9 @@
       <c r="A412" t="s">
         <v>38</v>
       </c>
+      <c r="B412" t="s">
+        <v>1</v>
+      </c>
       <c r="C412" t="s">
         <v>432</v>
       </c>
@@ -25087,6 +25312,9 @@
       <c r="A413" t="s">
         <v>38</v>
       </c>
+      <c r="B413" t="s">
+        <v>1</v>
+      </c>
       <c r="C413" t="s">
         <v>432</v>
       </c>
@@ -25110,6 +25338,9 @@
       <c r="A414" t="s">
         <v>38</v>
       </c>
+      <c r="B414" t="s">
+        <v>1</v>
+      </c>
       <c r="C414" t="s">
         <v>432</v>
       </c>
@@ -25133,6 +25364,9 @@
       <c r="A415" t="s">
         <v>38</v>
       </c>
+      <c r="B415" t="s">
+        <v>1</v>
+      </c>
       <c r="C415" t="s">
         <v>432</v>
       </c>
@@ -25156,6 +25390,9 @@
       <c r="A416" t="s">
         <v>38</v>
       </c>
+      <c r="B416" t="s">
+        <v>1</v>
+      </c>
       <c r="C416" t="s">
         <v>432</v>
       </c>
@@ -25179,6 +25416,9 @@
       <c r="A417" t="s">
         <v>38</v>
       </c>
+      <c r="B417" t="s">
+        <v>1</v>
+      </c>
       <c r="C417" t="s">
         <v>432</v>
       </c>
@@ -25200,6 +25440,9 @@
       <c r="A418" t="s">
         <v>38</v>
       </c>
+      <c r="B418" t="s">
+        <v>1</v>
+      </c>
       <c r="C418" t="s">
         <v>432</v>
       </c>
@@ -25221,6 +25464,9 @@
       <c r="A419" t="s">
         <v>38</v>
       </c>
+      <c r="B419" t="s">
+        <v>1</v>
+      </c>
       <c r="C419" t="s">
         <v>432</v>
       </c>
@@ -25242,6 +25488,9 @@
       <c r="A420" t="s">
         <v>38</v>
       </c>
+      <c r="B420" t="s">
+        <v>1</v>
+      </c>
       <c r="C420" t="s">
         <v>432</v>
       </c>
@@ -25263,6 +25512,9 @@
       <c r="A421" t="s">
         <v>38</v>
       </c>
+      <c r="B421" t="s">
+        <v>1</v>
+      </c>
       <c r="C421" t="s">
         <v>432</v>
       </c>
@@ -25284,6 +25536,9 @@
       <c r="A422" t="s">
         <v>38</v>
       </c>
+      <c r="B422" t="s">
+        <v>1</v>
+      </c>
       <c r="C422" t="s">
         <v>432</v>
       </c>
@@ -25304,6 +25559,9 @@
     <row r="423" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
         <v>38</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1</v>
       </c>
       <c r="C423" t="s">
         <v>432</v>

</xml_diff>

<commit_message>
Work on feed pars + regional diferentiation of max SNG
</commit_message>
<xml_diff>
--- a/data/prod_parameters/CattleHerd.xlsx
+++ b/data/prod_parameters/CattleHerd.xlsx
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3696" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3715" uniqueCount="543">
   <si>
     <t>value</t>
   </si>
@@ -1840,6 +1840,12 @@
   </si>
   <si>
     <t>Converted from ECM. 2013 kg ECM/cow/year</t>
+  </si>
+  <si>
+    <t>Ahlgren et al. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion</t>
+  </si>
+  <si>
+    <t>Växa Husdjursstatistik 2020, tab 32</t>
   </si>
 </sst>
 </file>
@@ -17926,6 +17932,7 @@
         <v>6</v>
       </c>
       <c r="I35">
+        <f>(27.5+28.4+27.6+29.9+30)/5</f>
         <v>28.68</v>
       </c>
       <c r="J35" t="s">
@@ -17933,6 +17940,9 @@
       </c>
       <c r="K35" t="s">
         <v>7</v>
+      </c>
+      <c r="L35" t="s">
+        <v>542</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -18578,6 +18588,9 @@
       <c r="K66" t="s">
         <v>10</v>
       </c>
+      <c r="L66" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
@@ -18598,6 +18611,9 @@
       <c r="K67" t="s">
         <v>22</v>
       </c>
+      <c r="L67" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
@@ -18618,6 +18634,9 @@
       <c r="K68" t="s">
         <v>24</v>
       </c>
+      <c r="L68" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
@@ -18638,6 +18657,9 @@
       <c r="K69" t="s">
         <v>22</v>
       </c>
+      <c r="L69" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -18658,6 +18680,9 @@
       <c r="K70" t="s">
         <v>24</v>
       </c>
+      <c r="L70" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
@@ -18678,6 +18703,9 @@
       <c r="K71" t="s">
         <v>28</v>
       </c>
+      <c r="L71" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
@@ -18698,6 +18726,9 @@
       <c r="K72" t="s">
         <v>24</v>
       </c>
+      <c r="L72" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
@@ -18718,6 +18749,9 @@
       <c r="K73" t="s">
         <v>28</v>
       </c>
+      <c r="L73" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
@@ -18737,6 +18771,9 @@
       </c>
       <c r="K74" t="s">
         <v>24</v>
+      </c>
+      <c r="L74" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
@@ -18774,6 +18811,9 @@
       <c r="K76" t="s">
         <v>10</v>
       </c>
+      <c r="L76" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
@@ -18794,6 +18834,9 @@
       <c r="K77" t="s">
         <v>22</v>
       </c>
+      <c r="L77" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
@@ -18814,6 +18857,9 @@
       <c r="K78" t="s">
         <v>39</v>
       </c>
+      <c r="L78" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
@@ -18834,6 +18880,9 @@
       <c r="K79" t="s">
         <v>22</v>
       </c>
+      <c r="L79" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
@@ -18854,6 +18903,9 @@
       <c r="K80" t="s">
         <v>39</v>
       </c>
+      <c r="L80" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
@@ -18874,6 +18926,9 @@
       <c r="K81" t="s">
         <v>28</v>
       </c>
+      <c r="L81" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
@@ -18894,6 +18949,9 @@
       <c r="K82" t="s">
         <v>39</v>
       </c>
+      <c r="L82" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
@@ -18914,6 +18972,9 @@
       <c r="K83" t="s">
         <v>28</v>
       </c>
+      <c r="L83" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
@@ -18933,6 +18994,9 @@
       </c>
       <c r="K84" t="s">
         <v>39</v>
+      </c>
+      <c r="L84" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>